<commit_message>
Update finance tracker with Elad's profile data
- Added army salary (1,462₪/month, 1st of month) and work salary placeholder (10th of month)
- Added fixed expenses: Claude AI (88₪), ChatGPT (71₪), Spotify (36₪), trainer Ofek Zarmati (600₪)
- Set monthly savings goal: 1,000₪
- Added budget plan and personalized financial tips
- Regenerated Excel workbook with updated data

https://claude.ai/code/session_01Cwu7SWtx13xhFUMhTaLvjR
</commit_message>
<xml_diff>
--- a/finance/מעקב_פיננסי.xlsx
+++ b/finance/מעקב_פיננסי.xlsx
@@ -25,7 +25,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="₪#,##0"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="26">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -104,6 +104,17 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="0027AE60"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="16"/>
@@ -123,14 +134,25 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="002980B9"/>
-      <sz val="12"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00E67E22"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="00E74C3C"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="002980B9"/>
+      <sz val="12"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -140,17 +162,6 @@
     <font>
       <name val="Calibri"/>
       <color rgb="0027AE60"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="0027AE60"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
@@ -166,7 +177,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="20">
     <fill>
       <patternFill/>
     </fill>
@@ -210,6 +221,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00F39C12"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="000D2137"/>
       </patternFill>
     </fill>
@@ -220,7 +236,27 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00071A0D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00051409"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00E67E22"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A1000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00130D00"/>
       </patternFill>
     </fill>
     <fill>
@@ -265,7 +301,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
@@ -313,13 +349,16 @@
     <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -334,82 +373,124 @@
     <xf numFmtId="0" fontId="12" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="14" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="13" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="14" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="164" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="22" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="23" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="14" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="9" fontId="21" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="13" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="22" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="23" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="14" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="9" fontId="21" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="13" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="18" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="9" fontId="17" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="18" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="25" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
   </cellXfs>
@@ -812,7 +893,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>עודכן לאחרונה: 17/04/2026 16:26</t>
+          <t>עודכן לאחרונה: 18/04/2026 05:35</t>
         </is>
       </c>
       <c r="Q2" s="2" t="n"/>
@@ -872,25 +953,25 @@
     <row r="5" ht="40" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>₪0</t>
+          <t>₪1,462</t>
         </is>
       </c>
       <c r="D5" s="2" t="n"/>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>₪0</t>
+          <t>₪795</t>
         </is>
       </c>
       <c r="H5" s="2" t="n"/>
       <c r="I5" s="10" t="inlineStr">
         <is>
-          <t>₪0</t>
+          <t>₪667</t>
         </is>
       </c>
       <c r="L5" s="2" t="n"/>
       <c r="M5" s="11" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>45.6%</t>
         </is>
       </c>
       <c r="P5" s="2" t="n"/>
@@ -924,7 +1005,7 @@
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="13" t="inlineStr">
         <is>
-          <t>ציון: 0/100  |  דורש שיפור 🔴</t>
+          <t>ציון: 35/100  |  דורש שיפור 🔴</t>
         </is>
       </c>
       <c r="Q8" s="2" t="n"/>
@@ -982,21 +1063,21 @@
         </is>
       </c>
       <c r="D12" s="2" t="n"/>
-      <c r="E12" s="16" t="inlineStr">
+      <c r="E12" s="17" t="inlineStr">
         <is>
-          <t>0/25</t>
+          <t>15/25</t>
         </is>
       </c>
       <c r="H12" s="2" t="n"/>
-      <c r="I12" s="16" t="inlineStr">
+      <c r="I12" s="17" t="inlineStr">
         <is>
-          <t>0/20</t>
+          <t>12/20</t>
         </is>
       </c>
       <c r="L12" s="2" t="n"/>
-      <c r="M12" s="16" t="inlineStr">
+      <c r="M12" s="17" t="inlineStr">
         <is>
-          <t>0/15</t>
+          <t>8/15</t>
         </is>
       </c>
       <c r="P12" s="2" t="n"/>
@@ -1026,7 +1107,7 @@
       <c r="S13" s="2" t="n"/>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="17" t="inlineStr">
+      <c r="A14" s="18" t="inlineStr">
         <is>
           <t>💡  טיפים פיננסיים אישיים</t>
         </is>
@@ -1036,9 +1117,9 @@
       <c r="S14" s="2" t="n"/>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="18" t="inlineStr">
+      <c r="A15" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ➤  הגדר תקציב חודשי לכל קטגוריה ועמוד בו</t>
+          <t xml:space="preserve">  ➤  ⚠️ הוצאות קבועות (795₪) = 54% מהכנסת הצבא בלבד — גבוה מאוד!</t>
         </is>
       </c>
       <c r="Q15" s="2" t="n"/>
@@ -1046,9 +1127,9 @@
       <c r="S15" s="2" t="n"/>
     </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="19" t="inlineStr">
+      <c r="A16" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ➤  שמור לפחות 3 חודשי הוצאות כקרן חירום</t>
+          <t xml:space="preserve">  ➤  💡 מטרת החיסכון שלך: 1,000₪/חודש — הגדר חשבון חיסכון נפרד והעבר אוטומטית</t>
         </is>
       </c>
       <c r="Q16" s="2" t="n"/>
@@ -1056,9 +1137,9 @@
       <c r="S16" s="2" t="n"/>
     </row>
     <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="18" t="inlineStr">
+      <c r="A17" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ➤  מטרה: לחסוך לפחות 20% מההכנסה נטו</t>
+          <t xml:space="preserve">  ➤  🤔 יש לך גם Claude וגם ChatGPT — חיסכון פוטנציאלי של 71₪/חודש</t>
         </is>
       </c>
       <c r="Q17" s="2" t="n"/>
@@ -1066,53 +1147,31 @@
       <c r="S17" s="2" t="n"/>
     </row>
     <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="19" t="inlineStr">
+      <c r="A18" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ➤  הגדל חיסכון אוטומטי ביום קבלת המשכורת</t>
+          <t xml:space="preserve">  ➤  💪 המאמן האישי (600₪) = 75% מסך ההוצאות הקבועות שלך — שקול אם זה משתלם</t>
         </is>
       </c>
       <c r="Q18" s="2" t="n"/>
       <c r="R18" s="2" t="n"/>
       <c r="S18" s="2" t="n"/>
     </row>
-    <row r="19">
-      <c r="A19" s="2" t="n"/>
-      <c r="B19" s="2" t="n"/>
-      <c r="C19" s="2" t="n"/>
-      <c r="D19" s="2" t="n"/>
-      <c r="E19" s="2" t="n"/>
-      <c r="F19" s="2" t="n"/>
-      <c r="G19" s="2" t="n"/>
-      <c r="H19" s="2" t="n"/>
-      <c r="I19" s="2" t="n"/>
-      <c r="J19" s="2" t="n"/>
-      <c r="K19" s="2" t="n"/>
-      <c r="L19" s="2" t="n"/>
-      <c r="M19" s="2" t="n"/>
-      <c r="N19" s="2" t="n"/>
-      <c r="O19" s="2" t="n"/>
-      <c r="P19" s="2" t="n"/>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ➤  📅 ביום קבלת משכורת — העבר מיד 1,000₪ לחיסכון לפני כל הוצאה אחרת</t>
+        </is>
+      </c>
       <c r="Q19" s="2" t="n"/>
       <c r="R19" s="2" t="n"/>
       <c r="S19" s="2" t="n"/>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="n"/>
-      <c r="B20" s="2" t="n"/>
-      <c r="C20" s="2" t="n"/>
-      <c r="D20" s="2" t="n"/>
-      <c r="E20" s="2" t="n"/>
-      <c r="F20" s="2" t="n"/>
-      <c r="G20" s="2" t="n"/>
-      <c r="H20" s="2" t="n"/>
-      <c r="I20" s="2" t="n"/>
-      <c r="J20" s="2" t="n"/>
-      <c r="K20" s="2" t="n"/>
-      <c r="L20" s="2" t="n"/>
-      <c r="M20" s="2" t="n"/>
-      <c r="N20" s="2" t="n"/>
-      <c r="O20" s="2" t="n"/>
-      <c r="P20" s="2" t="n"/>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ➤  🎯 לאחר עדכון כל ההוצאות הנוכחיות, נבנה תקציב מדויק יחד</t>
+        </is>
+      </c>
       <c r="Q20" s="2" t="n"/>
       <c r="R20" s="2" t="n"/>
       <c r="S20" s="2" t="n"/>
@@ -1937,15 +1996,17 @@
       <c r="S59" s="2" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="30">
+  <mergeCells count="32">
     <mergeCell ref="M11:O11"/>
     <mergeCell ref="A14:P14"/>
     <mergeCell ref="A17:P17"/>
     <mergeCell ref="I12:K12"/>
+    <mergeCell ref="A20:P20"/>
     <mergeCell ref="A12:C12"/>
     <mergeCell ref="M6:O6"/>
     <mergeCell ref="M12:O12"/>
     <mergeCell ref="E6:G6"/>
+    <mergeCell ref="A19:P19"/>
     <mergeCell ref="A10:P10"/>
     <mergeCell ref="E11:G11"/>
     <mergeCell ref="A5:C5"/>
@@ -1993,7 +2054,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1">
-      <c r="A1" s="20" t="inlineStr">
+      <c r="A1" s="21" t="inlineStr">
         <is>
           <t>📅  סיכום חודשי - הכנסות והוצאות</t>
         </is>
@@ -2016,37 +2077,37 @@
       <c r="N2" s="2" t="n"/>
     </row>
     <row r="3" ht="28" customHeight="1">
-      <c r="A3" s="21" t="inlineStr">
+      <c r="A3" s="22" t="inlineStr">
         <is>
           <t>חודש</t>
         </is>
       </c>
-      <c r="B3" s="21" t="inlineStr">
+      <c r="B3" s="22" t="inlineStr">
         <is>
           <t>הכנסה</t>
         </is>
       </c>
-      <c r="C3" s="21" t="inlineStr">
+      <c r="C3" s="22" t="inlineStr">
         <is>
           <t>הוצאות</t>
         </is>
       </c>
-      <c r="D3" s="21" t="inlineStr">
+      <c r="D3" s="22" t="inlineStr">
         <is>
           <t>חיסכון</t>
         </is>
       </c>
-      <c r="E3" s="21" t="inlineStr">
+      <c r="E3" s="22" t="inlineStr">
         <is>
           <t>% חיסכון</t>
         </is>
       </c>
-      <c r="F3" s="21" t="inlineStr">
+      <c r="F3" s="22" t="inlineStr">
         <is>
           <t>ציון</t>
         </is>
       </c>
-      <c r="G3" s="21" t="inlineStr">
+      <c r="G3" s="22" t="inlineStr">
         <is>
           <t>הערות</t>
         </is>
@@ -2092,39 +2153,39 @@
       <c r="N5" s="2" t="n"/>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="22" t="inlineStr">
+      <c r="A6" s="23" t="inlineStr">
         <is>
           <t>💵  מקורות הכנסה</t>
         </is>
       </c>
     </row>
     <row r="7" ht="25" customHeight="1">
-      <c r="A7" s="23" t="inlineStr">
+      <c r="A7" s="24" t="inlineStr">
         <is>
           <t>מקור הכנסה</t>
         </is>
       </c>
-      <c r="B7" s="23" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>סכום נטו</t>
         </is>
       </c>
-      <c r="C7" s="23" t="inlineStr">
+      <c r="C7" s="24" t="inlineStr">
         <is>
           <t>סכום ברוטו</t>
         </is>
       </c>
-      <c r="D7" s="23" t="inlineStr">
+      <c r="D7" s="24" t="inlineStr">
         <is>
           <t>תאריך קבלה</t>
         </is>
       </c>
-      <c r="E7" s="23" t="inlineStr">
+      <c r="E7" s="24" t="inlineStr">
         <is>
           <t>קבוע/משתנה</t>
         </is>
       </c>
-      <c r="F7" s="23" t="inlineStr">
+      <c r="F7" s="24" t="inlineStr">
         <is>
           <t>הערות</t>
         </is>
@@ -2138,13 +2199,33 @@
       <c r="M7" s="2" t="n"/>
       <c r="N7" s="2" t="n"/>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="n"/>
-      <c r="B8" s="2" t="n"/>
-      <c r="C8" s="2" t="n"/>
-      <c r="D8" s="2" t="n"/>
-      <c r="E8" s="2" t="n"/>
-      <c r="F8" s="2" t="n"/>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="25" t="inlineStr">
+        <is>
+          <t>צבא</t>
+        </is>
+      </c>
+      <c r="B8" s="26" t="n">
+        <v>1462</v>
+      </c>
+      <c r="C8" s="27" t="n">
+        <v>1462</v>
+      </c>
+      <c r="D8" s="25" t="inlineStr">
+        <is>
+          <t>1 לחודש</t>
+        </is>
+      </c>
+      <c r="E8" s="25" t="inlineStr">
+        <is>
+          <t>קבוע</t>
+        </is>
+      </c>
+      <c r="F8" s="25" t="inlineStr">
+        <is>
+          <t>שכר חייל קבוע</t>
+        </is>
+      </c>
       <c r="G8" s="2" t="n"/>
       <c r="H8" s="2" t="n"/>
       <c r="I8" s="2" t="n"/>
@@ -2154,13 +2235,33 @@
       <c r="M8" s="2" t="n"/>
       <c r="N8" s="2" t="n"/>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="n"/>
-      <c r="B9" s="2" t="n"/>
-      <c r="C9" s="2" t="n"/>
-      <c r="D9" s="2" t="n"/>
-      <c r="E9" s="2" t="n"/>
-      <c r="F9" s="2" t="n"/>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="28" t="inlineStr">
+        <is>
+          <t>עבודה</t>
+        </is>
+      </c>
+      <c r="B9" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="28" t="inlineStr">
+        <is>
+          <t>10 לחודש</t>
+        </is>
+      </c>
+      <c r="E9" s="28" t="inlineStr">
+        <is>
+          <t>קבוע</t>
+        </is>
+      </c>
+      <c r="F9" s="28" t="inlineStr">
+        <is>
+          <t>⚠️ לעדכן סכום</t>
+        </is>
+      </c>
       <c r="G9" s="2" t="n"/>
       <c r="H9" s="2" t="n"/>
       <c r="I9" s="2" t="n"/>
@@ -3639,44 +3740,44 @@
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1">
-      <c r="A1" s="24" t="inlineStr">
+      <c r="A1" s="31" t="inlineStr">
         <is>
           <t>💸  יומן הוצאות מפורט</t>
         </is>
       </c>
     </row>
     <row r="2" ht="26" customHeight="1">
-      <c r="A2" s="25" t="inlineStr">
+      <c r="A2" s="32" t="inlineStr">
         <is>
           <t>תאריך</t>
         </is>
       </c>
-      <c r="B2" s="25" t="inlineStr">
+      <c r="B2" s="32" t="inlineStr">
         <is>
           <t>קטגוריה</t>
         </is>
       </c>
-      <c r="C2" s="25" t="inlineStr">
+      <c r="C2" s="32" t="inlineStr">
         <is>
           <t>תיאור</t>
         </is>
       </c>
-      <c r="D2" s="25" t="inlineStr">
+      <c r="D2" s="32" t="inlineStr">
         <is>
           <t>סכום</t>
         </is>
       </c>
-      <c r="E2" s="25" t="inlineStr">
+      <c r="E2" s="32" t="inlineStr">
         <is>
           <t>שיטת תשלום</t>
         </is>
       </c>
-      <c r="F2" s="25" t="inlineStr">
+      <c r="F2" s="32" t="inlineStr">
         <is>
           <t>האם הכרחי?</t>
         </is>
       </c>
-      <c r="G2" s="25" t="inlineStr">
+      <c r="G2" s="32" t="inlineStr">
         <is>
           <t>הערות</t>
         </is>
@@ -10176,7 +10277,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1">
-      <c r="A1" s="26" t="inlineStr">
+      <c r="A1" s="33" t="inlineStr">
         <is>
           <t>📋  הוצאות קבועות חודשיות</t>
         </is>
@@ -10184,42 +10285,42 @@
       <c r="K1" s="2" t="n"/>
     </row>
     <row r="2" ht="26" customHeight="1">
-      <c r="A2" s="27" t="inlineStr">
+      <c r="A2" s="34" t="inlineStr">
         <is>
           <t>הוצאה</t>
         </is>
       </c>
-      <c r="B2" s="27" t="inlineStr">
+      <c r="B2" s="34" t="inlineStr">
         <is>
           <t>קטגוריה</t>
         </is>
       </c>
-      <c r="C2" s="27" t="inlineStr">
+      <c r="C2" s="34" t="inlineStr">
         <is>
           <t>סכום</t>
         </is>
       </c>
-      <c r="D2" s="27" t="inlineStr">
+      <c r="D2" s="34" t="inlineStr">
         <is>
           <t>יום חיוב</t>
         </is>
       </c>
-      <c r="E2" s="27" t="inlineStr">
+      <c r="E2" s="34" t="inlineStr">
         <is>
           <t>שיטת תשלום</t>
         </is>
       </c>
-      <c r="F2" s="27" t="inlineStr">
+      <c r="F2" s="34" t="inlineStr">
         <is>
           <t>חיוני?</t>
         </is>
       </c>
-      <c r="G2" s="27" t="inlineStr">
+      <c r="G2" s="34" t="inlineStr">
         <is>
           <t>אפשרי לחסוך?</t>
         </is>
       </c>
-      <c r="H2" s="27" t="inlineStr">
+      <c r="H2" s="34" t="inlineStr">
         <is>
           <t>הערות</t>
         </is>
@@ -10228,67 +10329,187 @@
       <c r="J2" s="2" t="n"/>
       <c r="K2" s="2" t="n"/>
     </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="28" t="inlineStr">
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="35" t="inlineStr">
+        <is>
+          <t>מנוי Claude AI</t>
+        </is>
+      </c>
+      <c r="B3" s="36" t="inlineStr">
+        <is>
+          <t>חשבונות קבועים</t>
+        </is>
+      </c>
+      <c r="C3" s="37" t="n">
+        <v>88</v>
+      </c>
+      <c r="D3" s="38" t="inlineStr">
+        <is>
+          <t>חודשי</t>
+        </is>
+      </c>
+      <c r="E3" s="38" t="inlineStr">
+        <is>
+          <t>כרטיס אשראי</t>
+        </is>
+      </c>
+      <c r="F3" s="38" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G3" s="38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H3" s="38" t="inlineStr">
+        <is>
+          <t>עוזר פיננסי + AI</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="n"/>
+      <c r="J3" s="2" t="n"/>
+      <c r="K3" s="2" t="n"/>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="39" t="inlineStr">
+        <is>
+          <t>מנוי ChatGPT</t>
+        </is>
+      </c>
+      <c r="B4" s="40" t="inlineStr">
+        <is>
+          <t>חשבונות קבועים</t>
+        </is>
+      </c>
+      <c r="C4" s="41" t="n">
+        <v>71</v>
+      </c>
+      <c r="D4" s="42" t="inlineStr">
+        <is>
+          <t>חודשי</t>
+        </is>
+      </c>
+      <c r="E4" s="42" t="inlineStr">
+        <is>
+          <t>כרטיס אשראי</t>
+        </is>
+      </c>
+      <c r="F4" s="42" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="G4" s="42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H4" s="42" t="inlineStr">
+        <is>
+          <t>בדוק האם נחוץ ביחד עם Claude</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="n"/>
+      <c r="J4" s="2" t="n"/>
+      <c r="K4" s="2" t="n"/>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="35" t="inlineStr">
+        <is>
+          <t>מנוי Spotify</t>
+        </is>
+      </c>
+      <c r="B5" s="36" t="inlineStr">
+        <is>
+          <t>חשבונות קבועים</t>
+        </is>
+      </c>
+      <c r="C5" s="37" t="n">
+        <v>36</v>
+      </c>
+      <c r="D5" s="38" t="inlineStr">
+        <is>
+          <t>חודשי</t>
+        </is>
+      </c>
+      <c r="E5" s="38" t="inlineStr">
+        <is>
+          <t>כרטיס אשראי</t>
+        </is>
+      </c>
+      <c r="F5" s="38" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="G5" s="38" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H5" s="38" t="inlineStr">
+        <is>
+          <t>מוזיקה</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="n"/>
+      <c r="J5" s="2" t="n"/>
+      <c r="K5" s="2" t="n"/>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="39" t="inlineStr">
+        <is>
+          <t>מאמן כושר - אופק זרמטי</t>
+        </is>
+      </c>
+      <c r="B6" s="40" t="inlineStr">
+        <is>
+          <t>ספורט</t>
+        </is>
+      </c>
+      <c r="C6" s="41" t="n">
+        <v>600</v>
+      </c>
+      <c r="D6" s="42" t="inlineStr">
+        <is>
+          <t>חודשי</t>
+        </is>
+      </c>
+      <c r="E6" s="42" t="inlineStr">
+        <is>
+          <t>העברה בנקאית</t>
+        </is>
+      </c>
+      <c r="F6" s="42" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="G6" s="42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H6" s="42" t="inlineStr">
+        <is>
+          <t>אימון אישי</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="n"/>
+      <c r="J6" s="2" t="n"/>
+      <c r="K6" s="2" t="n"/>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="43" t="inlineStr">
         <is>
           <t>סה"כ הוצאות קבועות</t>
         </is>
       </c>
-      <c r="C3" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n"/>
-      <c r="G3" s="2" t="n"/>
-      <c r="H3" s="2" t="n"/>
-      <c r="I3" s="2" t="n"/>
-      <c r="J3" s="2" t="n"/>
-      <c r="K3" s="2" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n"/>
-      <c r="B4" s="2" t="n"/>
-      <c r="C4" s="2" t="n"/>
-      <c r="D4" s="2" t="n"/>
-      <c r="E4" s="2" t="n"/>
-      <c r="F4" s="2" t="n"/>
-      <c r="G4" s="2" t="n"/>
-      <c r="H4" s="2" t="n"/>
-      <c r="I4" s="2" t="n"/>
-      <c r="J4" s="2" t="n"/>
-      <c r="K4" s="2" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n"/>
-      <c r="B5" s="2" t="n"/>
-      <c r="C5" s="2" t="n"/>
-      <c r="D5" s="2" t="n"/>
-      <c r="E5" s="2" t="n"/>
-      <c r="F5" s="2" t="n"/>
-      <c r="G5" s="2" t="n"/>
-      <c r="H5" s="2" t="n"/>
-      <c r="I5" s="2" t="n"/>
-      <c r="J5" s="2" t="n"/>
-      <c r="K5" s="2" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n"/>
-      <c r="B6" s="2" t="n"/>
-      <c r="C6" s="2" t="n"/>
-      <c r="D6" s="2" t="n"/>
-      <c r="E6" s="2" t="n"/>
-      <c r="F6" s="2" t="n"/>
-      <c r="G6" s="2" t="n"/>
-      <c r="H6" s="2" t="n"/>
-      <c r="I6" s="2" t="n"/>
-      <c r="J6" s="2" t="n"/>
-      <c r="K6" s="2" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n"/>
-      <c r="B7" s="2" t="n"/>
-      <c r="C7" s="2" t="n"/>
+      <c r="C7" s="44" t="n">
+        <v>795</v>
+      </c>
       <c r="D7" s="2" t="n"/>
       <c r="E7" s="2" t="n"/>
       <c r="F7" s="2" t="n"/>
@@ -11237,7 +11458,7 @@
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A7:B7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11262,7 +11483,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1">
-      <c r="A1" s="30" t="inlineStr">
+      <c r="A1" s="45" t="inlineStr">
         <is>
           <t>🎯  תוכנית תקציב חודשית</t>
         </is>
@@ -11270,32 +11491,32 @@
       <c r="K1" s="2" t="n"/>
     </row>
     <row r="2" ht="26" customHeight="1">
-      <c r="A2" s="31" t="inlineStr">
+      <c r="A2" s="46" t="inlineStr">
         <is>
           <t>קטגוריה</t>
         </is>
       </c>
-      <c r="B2" s="31" t="inlineStr">
+      <c r="B2" s="46" t="inlineStr">
         <is>
           <t>תקציב מתוכנן</t>
         </is>
       </c>
-      <c r="C2" s="31" t="inlineStr">
+      <c r="C2" s="46" t="inlineStr">
         <is>
           <t>הוצאה בפועל</t>
         </is>
       </c>
-      <c r="D2" s="31" t="inlineStr">
+      <c r="D2" s="46" t="inlineStr">
         <is>
           <t>הפרש</t>
         </is>
       </c>
-      <c r="E2" s="31" t="inlineStr">
+      <c r="E2" s="46" t="inlineStr">
         <is>
           <t>% ניצול</t>
         </is>
       </c>
-      <c r="F2" s="31" t="inlineStr">
+      <c r="F2" s="46" t="inlineStr">
         <is>
           <t>סטטוס</t>
         </is>
@@ -11307,24 +11528,24 @@
       <c r="K2" s="2" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="32" t="inlineStr">
+      <c r="A3" s="47" t="inlineStr">
         <is>
           <t>🛒 מזון וסופר</t>
         </is>
       </c>
-      <c r="B3" s="33" t="n">
+      <c r="B3" s="48" t="n">
+        <v>350</v>
+      </c>
+      <c r="C3" s="49" t="n">
         <v>0</v>
       </c>
-      <c r="C3" s="34" t="n">
+      <c r="D3" s="50" t="n">
+        <v>350</v>
+      </c>
+      <c r="E3" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="D3" s="35" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" s="37" t="inlineStr">
+      <c r="F3" s="52" t="inlineStr">
         <is>
           <t>✅ בתקציב</t>
         </is>
@@ -11336,24 +11557,24 @@
       <c r="K3" s="2" t="n"/>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="38" t="inlineStr">
+      <c r="A4" s="53" t="inlineStr">
         <is>
           <t>☕ מסעדות וקפה</t>
         </is>
       </c>
-      <c r="B4" s="39" t="n">
+      <c r="B4" s="54" t="n">
+        <v>200</v>
+      </c>
+      <c r="C4" s="55" t="n">
         <v>0</v>
       </c>
-      <c r="C4" s="40" t="n">
+      <c r="D4" s="56" t="n">
+        <v>200</v>
+      </c>
+      <c r="E4" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="D4" s="41" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="37" t="inlineStr">
+      <c r="F4" s="52" t="inlineStr">
         <is>
           <t>✅ בתקציב</t>
         </is>
@@ -11365,24 +11586,24 @@
       <c r="K4" s="2" t="n"/>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="32" t="inlineStr">
+      <c r="A5" s="47" t="inlineStr">
         <is>
           <t>🚗 תחבורה</t>
         </is>
       </c>
-      <c r="B5" s="33" t="n">
+      <c r="B5" s="48" t="n">
+        <v>150</v>
+      </c>
+      <c r="C5" s="49" t="n">
         <v>0</v>
       </c>
-      <c r="C5" s="34" t="n">
+      <c r="D5" s="50" t="n">
+        <v>150</v>
+      </c>
+      <c r="E5" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="D5" s="35" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="37" t="inlineStr">
+      <c r="F5" s="52" t="inlineStr">
         <is>
           <t>✅ בתקציב</t>
         </is>
@@ -11394,24 +11615,24 @@
       <c r="K5" s="2" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="38" t="inlineStr">
+      <c r="A6" s="53" t="inlineStr">
         <is>
           <t>🎮 בילויים</t>
         </is>
       </c>
-      <c r="B6" s="39" t="n">
+      <c r="B6" s="54" t="n">
+        <v>150</v>
+      </c>
+      <c r="C6" s="55" t="n">
         <v>0</v>
       </c>
-      <c r="C6" s="40" t="n">
+      <c r="D6" s="56" t="n">
+        <v>150</v>
+      </c>
+      <c r="E6" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="D6" s="41" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="37" t="inlineStr">
+      <c r="F6" s="52" t="inlineStr">
         <is>
           <t>✅ בתקציב</t>
         </is>
@@ -11423,24 +11644,24 @@
       <c r="K6" s="2" t="n"/>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="32" t="inlineStr">
+      <c r="A7" s="47" t="inlineStr">
         <is>
           <t>🏥 בריאות ורפואה</t>
         </is>
       </c>
-      <c r="B7" s="33" t="n">
+      <c r="B7" s="48" t="n">
+        <v>80</v>
+      </c>
+      <c r="C7" s="49" t="n">
         <v>0</v>
       </c>
-      <c r="C7" s="34" t="n">
+      <c r="D7" s="50" t="n">
+        <v>80</v>
+      </c>
+      <c r="E7" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="D7" s="35" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="37" t="inlineStr">
+      <c r="F7" s="52" t="inlineStr">
         <is>
           <t>✅ בתקציב</t>
         </is>
@@ -11452,24 +11673,24 @@
       <c r="K7" s="2" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="38" t="inlineStr">
+      <c r="A8" s="53" t="inlineStr">
         <is>
           <t>👕 ביגוד והנעלה</t>
         </is>
       </c>
-      <c r="B8" s="39" t="n">
+      <c r="B8" s="54" t="n">
+        <v>100</v>
+      </c>
+      <c r="C8" s="55" t="n">
         <v>0</v>
       </c>
-      <c r="C8" s="40" t="n">
+      <c r="D8" s="56" t="n">
+        <v>100</v>
+      </c>
+      <c r="E8" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="D8" s="41" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="37" t="inlineStr">
+      <c r="F8" s="52" t="inlineStr">
         <is>
           <t>✅ בתקציב</t>
         </is>
@@ -11481,24 +11702,24 @@
       <c r="K8" s="2" t="n"/>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="32" t="inlineStr">
+      <c r="A9" s="47" t="inlineStr">
         <is>
           <t>📋 חשבונות קבועים</t>
         </is>
       </c>
-      <c r="B9" s="33" t="n">
+      <c r="B9" s="48" t="n">
+        <v>195</v>
+      </c>
+      <c r="C9" s="49" t="n">
         <v>0</v>
       </c>
-      <c r="C9" s="34" t="n">
+      <c r="D9" s="50" t="n">
+        <v>195</v>
+      </c>
+      <c r="E9" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="D9" s="35" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="37" t="inlineStr">
+      <c r="F9" s="52" t="inlineStr">
         <is>
           <t>✅ בתקציב</t>
         </is>
@@ -11510,24 +11731,24 @@
       <c r="K9" s="2" t="n"/>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="38" t="inlineStr">
+      <c r="A10" s="53" t="inlineStr">
         <is>
           <t>🏠 שכר דירה</t>
         </is>
       </c>
-      <c r="B10" s="39" t="n">
+      <c r="B10" s="54" t="n">
         <v>0</v>
       </c>
-      <c r="C10" s="40" t="n">
+      <c r="C10" s="55" t="n">
         <v>0</v>
       </c>
-      <c r="D10" s="41" t="n">
+      <c r="D10" s="56" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="42" t="n">
+      <c r="E10" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="F10" s="37" t="inlineStr">
+      <c r="F10" s="52" t="inlineStr">
         <is>
           <t>✅ בתקציב</t>
         </is>
@@ -11539,24 +11760,24 @@
       <c r="K10" s="2" t="n"/>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="32" t="inlineStr">
+      <c r="A11" s="47" t="inlineStr">
         <is>
           <t>📚 חינוך</t>
         </is>
       </c>
-      <c r="B11" s="33" t="n">
+      <c r="B11" s="48" t="n">
         <v>0</v>
       </c>
-      <c r="C11" s="34" t="n">
+      <c r="C11" s="49" t="n">
         <v>0</v>
       </c>
-      <c r="D11" s="35" t="n">
+      <c r="D11" s="50" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="36" t="n">
+      <c r="E11" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="F11" s="37" t="inlineStr">
+      <c r="F11" s="52" t="inlineStr">
         <is>
           <t>✅ בתקציב</t>
         </is>
@@ -11568,24 +11789,24 @@
       <c r="K11" s="2" t="n"/>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="38" t="inlineStr">
+      <c r="A12" s="53" t="inlineStr">
         <is>
           <t>💪 ספורט</t>
         </is>
       </c>
-      <c r="B12" s="39" t="n">
+      <c r="B12" s="54" t="n">
+        <v>600</v>
+      </c>
+      <c r="C12" s="55" t="n">
         <v>0</v>
       </c>
-      <c r="C12" s="40" t="n">
+      <c r="D12" s="56" t="n">
+        <v>600</v>
+      </c>
+      <c r="E12" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="D12" s="41" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="37" t="inlineStr">
+      <c r="F12" s="52" t="inlineStr">
         <is>
           <t>✅ בתקציב</t>
         </is>
@@ -11597,24 +11818,24 @@
       <c r="K12" s="2" t="n"/>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="32" t="inlineStr">
+      <c r="A13" s="47" t="inlineStr">
         <is>
           <t>🎁 מתנות</t>
         </is>
       </c>
-      <c r="B13" s="33" t="n">
+      <c r="B13" s="48" t="n">
+        <v>50</v>
+      </c>
+      <c r="C13" s="49" t="n">
         <v>0</v>
       </c>
-      <c r="C13" s="34" t="n">
+      <c r="D13" s="50" t="n">
+        <v>50</v>
+      </c>
+      <c r="E13" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="D13" s="35" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="37" t="inlineStr">
+      <c r="F13" s="52" t="inlineStr">
         <is>
           <t>✅ בתקציב</t>
         </is>
@@ -11626,24 +11847,24 @@
       <c r="K13" s="2" t="n"/>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="38" t="inlineStr">
+      <c r="A14" s="53" t="inlineStr">
         <is>
           <t>💰 חיסכון</t>
         </is>
       </c>
-      <c r="B14" s="39" t="n">
+      <c r="B14" s="54" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C14" s="55" t="n">
         <v>0</v>
       </c>
-      <c r="C14" s="40" t="n">
+      <c r="D14" s="56" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E14" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="D14" s="41" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" s="37" t="inlineStr">
+      <c r="F14" s="52" t="inlineStr">
         <is>
           <t>✅ בתקציב</t>
         </is>
@@ -11655,24 +11876,24 @@
       <c r="K14" s="2" t="n"/>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="32" t="inlineStr">
+      <c r="A15" s="47" t="inlineStr">
         <is>
           <t>📈 השקעות</t>
         </is>
       </c>
-      <c r="B15" s="33" t="n">
+      <c r="B15" s="48" t="n">
         <v>0</v>
       </c>
-      <c r="C15" s="34" t="n">
+      <c r="C15" s="49" t="n">
         <v>0</v>
       </c>
-      <c r="D15" s="35" t="n">
+      <c r="D15" s="50" t="n">
         <v>0</v>
       </c>
-      <c r="E15" s="36" t="n">
+      <c r="E15" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="F15" s="37" t="inlineStr">
+      <c r="F15" s="52" t="inlineStr">
         <is>
           <t>✅ בתקציב</t>
         </is>
@@ -11684,24 +11905,24 @@
       <c r="K15" s="2" t="n"/>
     </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="38" t="inlineStr">
+      <c r="A16" s="53" t="inlineStr">
         <is>
           <t>💳 אחר</t>
         </is>
       </c>
-      <c r="B16" s="39" t="n">
+      <c r="B16" s="54" t="n">
+        <v>100</v>
+      </c>
+      <c r="C16" s="55" t="n">
         <v>0</v>
       </c>
-      <c r="C16" s="40" t="n">
+      <c r="D16" s="56" t="n">
+        <v>100</v>
+      </c>
+      <c r="E16" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="D16" s="41" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="37" t="inlineStr">
+      <c r="F16" s="52" t="inlineStr">
         <is>
           <t>✅ בתקציב</t>
         </is>
@@ -12558,39 +12779,39 @@
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1">
-      <c r="A1" s="43" t="inlineStr">
+      <c r="A1" s="58" t="inlineStr">
         <is>
           <t>📈  ניתוח הוצאות לפי קטגוריות</t>
         </is>
       </c>
     </row>
     <row r="2" ht="26" customHeight="1">
-      <c r="A2" s="44" t="inlineStr">
+      <c r="A2" s="59" t="inlineStr">
         <is>
           <t>קטגוריה</t>
         </is>
       </c>
-      <c r="B2" s="44" t="inlineStr">
+      <c r="B2" s="59" t="inlineStr">
         <is>
           <t>סה"כ החודש</t>
         </is>
       </c>
-      <c r="C2" s="44" t="inlineStr">
+      <c r="C2" s="59" t="inlineStr">
         <is>
           <t>% מסה"כ</t>
         </is>
       </c>
-      <c r="D2" s="44" t="inlineStr">
+      <c r="D2" s="59" t="inlineStr">
         <is>
           <t>ממוצע יומי</t>
         </is>
       </c>
-      <c r="E2" s="44" t="inlineStr">
+      <c r="E2" s="59" t="inlineStr">
         <is>
           <t>מספר עסקאות</t>
         </is>
       </c>
-      <c r="F2" s="44" t="inlineStr">
+      <c r="F2" s="59" t="inlineStr">
         <is>
           <t>הכי גבוה</t>
         </is>
@@ -12605,15 +12826,15 @@
       <c r="N2" s="2" t="n"/>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="45" t="inlineStr">
+      <c r="A3" s="60" t="inlineStr">
         <is>
           <t>סה"כ</t>
         </is>
       </c>
-      <c r="B3" s="46" t="n">
+      <c r="B3" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="C3" s="47" t="n">
+      <c r="C3" s="62" t="n">
         <v>1</v>
       </c>
       <c r="D3" s="2" t="n"/>
@@ -13878,69 +14099,69 @@
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1">
-      <c r="A1" s="48" t="inlineStr">
+      <c r="A1" s="63" t="inlineStr">
         <is>
           <t>📄  יומן תלושי שכר</t>
         </is>
       </c>
     </row>
     <row r="2" ht="26" customHeight="1">
-      <c r="A2" s="49" t="inlineStr">
+      <c r="A2" s="64" t="inlineStr">
         <is>
           <t>חודש</t>
         </is>
       </c>
-      <c r="B2" s="49" t="inlineStr">
+      <c r="B2" s="64" t="inlineStr">
         <is>
           <t>מעסיק</t>
         </is>
       </c>
-      <c r="C2" s="49" t="inlineStr">
+      <c r="C2" s="64" t="inlineStr">
         <is>
           <t>ברוטו</t>
         </is>
       </c>
-      <c r="D2" s="49" t="inlineStr">
+      <c r="D2" s="64" t="inlineStr">
         <is>
           <t>נטו</t>
         </is>
       </c>
-      <c r="E2" s="49" t="inlineStr">
+      <c r="E2" s="64" t="inlineStr">
         <is>
           <t>מס הכנסה</t>
         </is>
       </c>
-      <c r="F2" s="49" t="inlineStr">
+      <c r="F2" s="64" t="inlineStr">
         <is>
           <t>ביטוח לאומי</t>
         </is>
       </c>
-      <c r="G2" s="49" t="inlineStr">
+      <c r="G2" s="64" t="inlineStr">
         <is>
           <t>בריאות</t>
         </is>
       </c>
-      <c r="H2" s="49" t="inlineStr">
+      <c r="H2" s="64" t="inlineStr">
         <is>
           <t>קרן פנסיה</t>
         </is>
       </c>
-      <c r="I2" s="49" t="inlineStr">
+      <c r="I2" s="64" t="inlineStr">
         <is>
           <t>קרן השתלמות</t>
         </is>
       </c>
-      <c r="J2" s="49" t="inlineStr">
+      <c r="J2" s="64" t="inlineStr">
         <is>
           <t>נסיעות</t>
         </is>
       </c>
-      <c r="K2" s="49" t="inlineStr">
+      <c r="K2" s="64" t="inlineStr">
         <is>
           <t>שעות נוספות</t>
         </is>
       </c>
-      <c r="L2" s="49" t="inlineStr">
+      <c r="L2" s="64" t="inlineStr">
         <is>
           <t>הערות</t>
         </is>

</xml_diff>

<commit_message>
Add April 2026 full financial data for Elad
- Income: army 1,462₪ + work 5,616₪ + one-time from mom 2,000₪ = 9,078₪
- 30 expense transactions categorized across 10 categories
- Total expenses: 5,082₪ | Net savings: 3,996₪
- Health score: 60/100
- Balance: 4,114₪ bank + 600₪ cash = 4,714₪
- Personalized tips based on spending patterns

https://claude.ai/code/session_01Cwu7SWtx13xhFUMhTaLvjR
</commit_message>
<xml_diff>
--- a/finance/מעקב_פיננסי.xlsx
+++ b/finance/מעקב_פיננסי.xlsx
@@ -22,10 +22,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="₪#,##0"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="₪#,##0.0"/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="34">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -92,6 +94,22 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="0027AE60"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="13"/>
@@ -101,11 +119,6 @@
       <b val="1"/>
       <color rgb="0027AE60"/>
       <sz val="12"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -127,18 +140,6 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00E67E22"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
       <color rgb="00E67E22"/>
       <sz val="11"/>
     </font>
@@ -147,6 +148,17 @@
       <b val="1"/>
       <color rgb="00E74C3C"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00F39C12"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00E67E22"/>
+      <sz val="12"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -161,7 +173,7 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="0027AE60"/>
+      <color rgb="00E74C3C"/>
       <sz val="11"/>
     </font>
     <font>
@@ -173,11 +185,47 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="002980B9"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00E67E22"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="008E44AD"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="0017A589"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00F39C12"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000F3460"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="0017A589"/>
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="20">
+  <fills count="24">
     <fill>
       <patternFill/>
     </fill>
@@ -246,6 +294,16 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00200A0A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00180707"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00E67E22"/>
       </patternFill>
     </fill>
@@ -267,6 +325,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00000B15"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000A001A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00070014"/>
       </patternFill>
     </fill>
     <fill>
@@ -301,7 +369,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="104">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
@@ -337,13 +405,16 @@
     <xf numFmtId="0" fontId="5" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -367,43 +438,64 @@
     <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="11" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="12" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="11" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="16" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="11" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="16" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="11" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -412,85 +504,178 @@
     <xf numFmtId="164" fontId="20" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="20" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="164" fontId="22" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="20" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="9" fontId="13" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="14" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="164" fontId="22" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="24" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="9" fontId="13" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="25" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="20" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="11" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="24" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="9" fontId="18" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="25" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="20" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="11" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="22" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="27" fillId="22" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="22" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="22" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="22" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="22" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="28" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="29" fillId="22" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="30" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="22" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="31" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="32" fillId="22" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="9" fontId="13" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
   </cellXfs>
@@ -893,7 +1078,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>עודכן לאחרונה: 18/04/2026 05:35</t>
+          <t>עודכן לאחרונה: 18/04/2026 06:00</t>
         </is>
       </c>
       <c r="Q2" s="2" t="n"/>
@@ -953,25 +1138,25 @@
     <row r="5" ht="40" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>₪1,462</t>
+          <t>₪9,078</t>
         </is>
       </c>
       <c r="D5" s="2" t="n"/>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>₪795</t>
+          <t>₪5,082</t>
         </is>
       </c>
       <c r="H5" s="2" t="n"/>
       <c r="I5" s="10" t="inlineStr">
         <is>
-          <t>₪667</t>
+          <t>₪3,996</t>
         </is>
       </c>
       <c r="L5" s="2" t="n"/>
       <c r="M5" s="11" t="inlineStr">
         <is>
-          <t>45.6%</t>
+          <t>44.0%</t>
         </is>
       </c>
       <c r="P5" s="2" t="n"/>
@@ -1005,7 +1190,7 @@
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="13" t="inlineStr">
         <is>
-          <t>ציון: 35/100  |  דורש שיפור 🔴</t>
+          <t>ציון: 60/100  |  טוב 👍</t>
         </is>
       </c>
       <c r="Q8" s="2" t="n"/>
@@ -1059,25 +1244,25 @@
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="16" t="inlineStr">
         <is>
-          <t>0/30</t>
+          <t>27/30</t>
         </is>
       </c>
       <c r="D12" s="2" t="n"/>
       <c r="E12" s="17" t="inlineStr">
         <is>
-          <t>15/25</t>
+          <t>8/25</t>
         </is>
       </c>
       <c r="H12" s="2" t="n"/>
-      <c r="I12" s="17" t="inlineStr">
-        <is>
-          <t>12/20</t>
+      <c r="I12" s="16" t="inlineStr">
+        <is>
+          <t>16/20</t>
         </is>
       </c>
       <c r="L12" s="2" t="n"/>
-      <c r="M12" s="17" t="inlineStr">
-        <is>
-          <t>8/15</t>
+      <c r="M12" s="18" t="inlineStr">
+        <is>
+          <t>9/15</t>
         </is>
       </c>
       <c r="P12" s="2" t="n"/>
@@ -1107,7 +1292,7 @@
       <c r="S13" s="2" t="n"/>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="18" t="inlineStr">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>💡  טיפים פיננסיים אישיים</t>
         </is>
@@ -1117,9 +1302,9 @@
       <c r="S14" s="2" t="n"/>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ➤  ⚠️ הוצאות קבועות (795₪) = 54% מהכנסת הצבא בלבד — גבוה מאוד!</t>
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ➤  ⚠️ מסעדות + משלוחים: 811₪ ב-14 עסקאות! תקציב מומלץ: 200₪ — חיסכון פוטנציאלי: 611₪/חודש</t>
         </is>
       </c>
       <c r="Q15" s="2" t="n"/>
@@ -1127,9 +1312,9 @@
       <c r="S15" s="2" t="n"/>
     </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ➤  💡 מטרת החיסכון שלך: 1,000₪/חודש — הגדר חשבון חיסכון נפרד והעבר אוטומטית</t>
+      <c r="A16" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ➤  💝 מתנות לבת זוג החודש: 860₪ (תכשיט 415₪ + פרחים 345₪) — קבע תקציב מתנות: 200₪/חודש</t>
         </is>
       </c>
       <c r="Q16" s="2" t="n"/>
@@ -1137,9 +1322,9 @@
       <c r="S16" s="2" t="n"/>
     </row>
     <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ➤  🤔 יש לך גם Claude וגם ChatGPT — חיסכון פוטנציאלי של 71₪/חודש</t>
+      <c r="A17" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ➤  ⚡ 5 משקאות אנרגיה = 61₪ — קנה קרטון ב-45₪ וחסוך כמעט חצי</t>
         </is>
       </c>
       <c r="Q17" s="2" t="n"/>
@@ -1147,9 +1332,9 @@
       <c r="S17" s="2" t="n"/>
     </row>
     <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ➤  💪 המאמן האישי (600₪) = 75% מסך ההוצאות הקבועות שלך — שקול אם זה משתלם</t>
+      <c r="A18" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ➤  💡 Claude + ChatGPT = 159₪/חודש — יש לך כבר Claude כיועץ פיננסי, שקול לבטל ChatGPT</t>
         </is>
       </c>
       <c r="Q18" s="2" t="n"/>
@@ -1157,9 +1342,9 @@
       <c r="S18" s="2" t="n"/>
     </row>
     <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ➤  📅 ביום קבלת משכורת — העבר מיד 1,000₪ לחיסכון לפני כל הוצאה אחרת</t>
+      <c r="A19" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ➤  🚗 שיעורי נהיגה: 1,100₪ — השקעה חשובה! ודא כמה שיעורים נותרו לבחינה</t>
         </is>
       </c>
       <c r="Q19" s="2" t="n"/>
@@ -1167,9 +1352,9 @@
       <c r="S19" s="2" t="n"/>
     </row>
     <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ➤  🎯 לאחר עדכון כל ההוצאות הנוכחיות, נבנה תקציב מדויק יחד</t>
+      <c r="A20" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ➤  💰 2,000₪ מאמא = חד פעמי! תכנן את מאי רק על בסיס 7,078₪ הכנסה קבועה</t>
         </is>
       </c>
       <c r="Q20" s="2" t="n"/>
@@ -2054,7 +2239,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1">
-      <c r="A1" s="21" t="inlineStr">
+      <c r="A1" s="22" t="inlineStr">
         <is>
           <t>📅  סיכום חודשי - הכנסות והוצאות</t>
         </is>
@@ -2077,37 +2262,37 @@
       <c r="N2" s="2" t="n"/>
     </row>
     <row r="3" ht="28" customHeight="1">
-      <c r="A3" s="22" t="inlineStr">
+      <c r="A3" s="23" t="inlineStr">
         <is>
           <t>חודש</t>
         </is>
       </c>
-      <c r="B3" s="22" t="inlineStr">
+      <c r="B3" s="23" t="inlineStr">
         <is>
           <t>הכנסה</t>
         </is>
       </c>
-      <c r="C3" s="22" t="inlineStr">
+      <c r="C3" s="23" t="inlineStr">
         <is>
           <t>הוצאות</t>
         </is>
       </c>
-      <c r="D3" s="22" t="inlineStr">
+      <c r="D3" s="23" t="inlineStr">
         <is>
           <t>חיסכון</t>
         </is>
       </c>
-      <c r="E3" s="22" t="inlineStr">
+      <c r="E3" s="23" t="inlineStr">
         <is>
           <t>% חיסכון</t>
         </is>
       </c>
-      <c r="F3" s="22" t="inlineStr">
+      <c r="F3" s="23" t="inlineStr">
         <is>
           <t>ציון</t>
         </is>
       </c>
-      <c r="G3" s="22" t="inlineStr">
+      <c r="G3" s="23" t="inlineStr">
         <is>
           <t>הערות</t>
         </is>
@@ -2120,14 +2305,32 @@
       <c r="M3" s="2" t="n"/>
       <c r="N3" s="2" t="n"/>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="n"/>
-      <c r="B4" s="2" t="n"/>
-      <c r="C4" s="2" t="n"/>
-      <c r="D4" s="2" t="n"/>
-      <c r="E4" s="2" t="n"/>
-      <c r="F4" s="2" t="n"/>
-      <c r="G4" s="2" t="n"/>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="24" t="inlineStr">
+        <is>
+          <t>אפריל 2026</t>
+        </is>
+      </c>
+      <c r="B4" s="25" t="n">
+        <v>9078</v>
+      </c>
+      <c r="C4" s="25" t="n">
+        <v>5082</v>
+      </c>
+      <c r="D4" s="26" t="n">
+        <v>3996</v>
+      </c>
+      <c r="E4" s="27" t="n">
+        <v>0.4401850627891606</v>
+      </c>
+      <c r="F4" s="28" t="n">
+        <v>60</v>
+      </c>
+      <c r="G4" s="24" t="inlineStr">
+        <is>
+          <t>הכנסה גבוהה: עבודה 5,616₪ + צבא 1,462₪ + אמא 2,000₪ (חד פעמי). הכנסה רגילה: 7,078₪</t>
+        </is>
+      </c>
       <c r="H4" s="2" t="n"/>
       <c r="I4" s="2" t="n"/>
       <c r="J4" s="2" t="n"/>
@@ -2152,78 +2355,58 @@
       <c r="M5" s="2" t="n"/>
       <c r="N5" s="2" t="n"/>
     </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="23" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="2" t="n"/>
+      <c r="B6" s="2" t="n"/>
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="n"/>
+      <c r="G6" s="2" t="n"/>
+      <c r="H6" s="2" t="n"/>
+      <c r="I6" s="2" t="n"/>
+      <c r="J6" s="2" t="n"/>
+      <c r="K6" s="2" t="n"/>
+      <c r="L6" s="2" t="n"/>
+      <c r="M6" s="2" t="n"/>
+      <c r="N6" s="2" t="n"/>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="29" t="inlineStr">
         <is>
           <t>💵  מקורות הכנסה</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="25" customHeight="1">
-      <c r="A7" s="24" t="inlineStr">
+    <row r="8" ht="25" customHeight="1">
+      <c r="A8" s="30" t="inlineStr">
         <is>
           <t>מקור הכנסה</t>
         </is>
       </c>
-      <c r="B7" s="24" t="inlineStr">
+      <c r="B8" s="30" t="inlineStr">
         <is>
           <t>סכום נטו</t>
         </is>
       </c>
-      <c r="C7" s="24" t="inlineStr">
+      <c r="C8" s="30" t="inlineStr">
         <is>
           <t>סכום ברוטו</t>
         </is>
       </c>
-      <c r="D7" s="24" t="inlineStr">
+      <c r="D8" s="30" t="inlineStr">
         <is>
           <t>תאריך קבלה</t>
         </is>
       </c>
-      <c r="E7" s="24" t="inlineStr">
+      <c r="E8" s="30" t="inlineStr">
         <is>
           <t>קבוע/משתנה</t>
         </is>
       </c>
-      <c r="F7" s="24" t="inlineStr">
+      <c r="F8" s="30" t="inlineStr">
         <is>
           <t>הערות</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="n"/>
-      <c r="H7" s="2" t="n"/>
-      <c r="I7" s="2" t="n"/>
-      <c r="J7" s="2" t="n"/>
-      <c r="K7" s="2" t="n"/>
-      <c r="L7" s="2" t="n"/>
-      <c r="M7" s="2" t="n"/>
-      <c r="N7" s="2" t="n"/>
-    </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="25" t="inlineStr">
-        <is>
-          <t>צבא</t>
-        </is>
-      </c>
-      <c r="B8" s="26" t="n">
-        <v>1462</v>
-      </c>
-      <c r="C8" s="27" t="n">
-        <v>1462</v>
-      </c>
-      <c r="D8" s="25" t="inlineStr">
-        <is>
-          <t>1 לחודש</t>
-        </is>
-      </c>
-      <c r="E8" s="25" t="inlineStr">
-        <is>
-          <t>קבוע</t>
-        </is>
-      </c>
-      <c r="F8" s="25" t="inlineStr">
-        <is>
-          <t>שכר חייל קבוע</t>
         </is>
       </c>
       <c r="G8" s="2" t="n"/>
@@ -2236,30 +2419,30 @@
       <c r="N8" s="2" t="n"/>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="28" t="inlineStr">
-        <is>
-          <t>עבודה</t>
-        </is>
-      </c>
-      <c r="B9" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="28" t="inlineStr">
-        <is>
-          <t>10 לחודש</t>
-        </is>
-      </c>
-      <c r="E9" s="28" t="inlineStr">
+      <c r="A9" s="31" t="inlineStr">
+        <is>
+          <t>צבא</t>
+        </is>
+      </c>
+      <c r="B9" s="32" t="n">
+        <v>1462</v>
+      </c>
+      <c r="C9" s="33" t="n">
+        <v>1462</v>
+      </c>
+      <c r="D9" s="31" t="inlineStr">
+        <is>
+          <t>1 לחודש</t>
+        </is>
+      </c>
+      <c r="E9" s="31" t="inlineStr">
         <is>
           <t>קבוע</t>
         </is>
       </c>
-      <c r="F9" s="28" t="inlineStr">
-        <is>
-          <t>⚠️ לעדכן סכום</t>
+      <c r="F9" s="31" t="inlineStr">
+        <is>
+          <t>שכר חייל קבוע</t>
         </is>
       </c>
       <c r="G9" s="2" t="n"/>
@@ -2271,13 +2454,33 @@
       <c r="M9" s="2" t="n"/>
       <c r="N9" s="2" t="n"/>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="n"/>
-      <c r="B10" s="2" t="n"/>
-      <c r="C10" s="2" t="n"/>
-      <c r="D10" s="2" t="n"/>
-      <c r="E10" s="2" t="n"/>
-      <c r="F10" s="2" t="n"/>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="34" t="inlineStr">
+        <is>
+          <t>עבודה</t>
+        </is>
+      </c>
+      <c r="B10" s="35" t="n">
+        <v>5616</v>
+      </c>
+      <c r="C10" s="36" t="n">
+        <v>5616</v>
+      </c>
+      <c r="D10" s="34" t="inlineStr">
+        <is>
+          <t>10 לחודש</t>
+        </is>
+      </c>
+      <c r="E10" s="34" t="inlineStr">
+        <is>
+          <t>קבוע</t>
+        </is>
+      </c>
+      <c r="F10" s="34" t="inlineStr">
+        <is>
+          <t>משכורת עבודה</t>
+        </is>
+      </c>
       <c r="G10" s="2" t="n"/>
       <c r="H10" s="2" t="n"/>
       <c r="I10" s="2" t="n"/>
@@ -2287,13 +2490,33 @@
       <c r="M10" s="2" t="n"/>
       <c r="N10" s="2" t="n"/>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="n"/>
-      <c r="B11" s="2" t="n"/>
-      <c r="C11" s="2" t="n"/>
-      <c r="D11" s="2" t="n"/>
-      <c r="E11" s="2" t="n"/>
-      <c r="F11" s="2" t="n"/>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="31" t="inlineStr">
+        <is>
+          <t>אמא - תוספת חד פעמית</t>
+        </is>
+      </c>
+      <c r="B11" s="32" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C11" s="33" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D11" s="31" t="inlineStr">
+        <is>
+          <t>אפריל 2026</t>
+        </is>
+      </c>
+      <c r="E11" s="31" t="inlineStr">
+        <is>
+          <t>חד פעמי</t>
+        </is>
+      </c>
+      <c r="F11" s="31" t="inlineStr">
+        <is>
+          <t>⚠️ לא לחשב כהכנסה קבועה לתכנון עתידי</t>
+        </is>
+      </c>
       <c r="G11" s="2" t="n"/>
       <c r="H11" s="2" t="n"/>
       <c r="I11" s="2" t="n"/>
@@ -3713,7 +3936,7 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A6:N6"/>
+    <mergeCell ref="A7:N7"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3740,44 +3963,44 @@
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1">
-      <c r="A1" s="31" t="inlineStr">
+      <c r="A1" s="37" t="inlineStr">
         <is>
           <t>💸  יומן הוצאות מפורט</t>
         </is>
       </c>
     </row>
     <row r="2" ht="26" customHeight="1">
-      <c r="A2" s="32" t="inlineStr">
+      <c r="A2" s="38" t="inlineStr">
         <is>
           <t>תאריך</t>
         </is>
       </c>
-      <c r="B2" s="32" t="inlineStr">
+      <c r="B2" s="38" t="inlineStr">
         <is>
           <t>קטגוריה</t>
         </is>
       </c>
-      <c r="C2" s="32" t="inlineStr">
+      <c r="C2" s="38" t="inlineStr">
         <is>
           <t>תיאור</t>
         </is>
       </c>
-      <c r="D2" s="32" t="inlineStr">
+      <c r="D2" s="38" t="inlineStr">
         <is>
           <t>סכום</t>
         </is>
       </c>
-      <c r="E2" s="32" t="inlineStr">
+      <c r="E2" s="38" t="inlineStr">
         <is>
           <t>שיטת תשלום</t>
         </is>
       </c>
-      <c r="F2" s="32" t="inlineStr">
+      <c r="F2" s="38" t="inlineStr">
         <is>
           <t>האם הכרחי?</t>
         </is>
       </c>
-      <c r="G2" s="32" t="inlineStr">
+      <c r="G2" s="38" t="inlineStr">
         <is>
           <t>הערות</t>
         </is>
@@ -3787,391 +4010,1075 @@
       <c r="J2" s="2" t="n"/>
       <c r="K2" s="2" t="n"/>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="n"/>
-      <c r="B3" s="2" t="n"/>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n"/>
-      <c r="G3" s="2" t="n"/>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="39" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="B3" s="40" t="inlineStr">
+        <is>
+          <t>מתנות</t>
+        </is>
+      </c>
+      <c r="C3" s="39" t="inlineStr">
+        <is>
+          <t>מתנה - זארה</t>
+        </is>
+      </c>
+      <c r="D3" s="41" t="n">
+        <v>100</v>
+      </c>
+      <c r="E3" s="39" t="inlineStr">
+        <is>
+          <t>לא צוין</t>
+        </is>
+      </c>
+      <c r="F3" s="42" t="inlineStr">
+        <is>
+          <t>❌ לא</t>
+        </is>
+      </c>
+      <c r="G3" s="39" t="inlineStr"/>
       <c r="H3" s="2" t="n"/>
       <c r="I3" s="2" t="n"/>
       <c r="J3" s="2" t="n"/>
       <c r="K3" s="2" t="n"/>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="n"/>
-      <c r="B4" s="2" t="n"/>
-      <c r="C4" s="2" t="n"/>
-      <c r="D4" s="2" t="n"/>
-      <c r="E4" s="2" t="n"/>
-      <c r="F4" s="2" t="n"/>
-      <c r="G4" s="2" t="n"/>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="43" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="B4" s="44" t="inlineStr">
+        <is>
+          <t>מתנות</t>
+        </is>
+      </c>
+      <c r="C4" s="43" t="inlineStr">
+        <is>
+          <t>תכשיט מגנוליה לבת זוג</t>
+        </is>
+      </c>
+      <c r="D4" s="45" t="n">
+        <v>415</v>
+      </c>
+      <c r="E4" s="43" t="inlineStr">
+        <is>
+          <t>לא צוין</t>
+        </is>
+      </c>
+      <c r="F4" s="46" t="inlineStr">
+        <is>
+          <t>❌ לא</t>
+        </is>
+      </c>
+      <c r="G4" s="43" t="inlineStr">
+        <is>
+          <t>רכישה גדולה</t>
+        </is>
+      </c>
       <c r="H4" s="2" t="n"/>
       <c r="I4" s="2" t="n"/>
       <c r="J4" s="2" t="n"/>
       <c r="K4" s="2" t="n"/>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="n"/>
-      <c r="B5" s="2" t="n"/>
-      <c r="C5" s="2" t="n"/>
-      <c r="D5" s="2" t="n"/>
-      <c r="E5" s="2" t="n"/>
-      <c r="F5" s="2" t="n"/>
-      <c r="G5" s="2" t="n"/>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="39" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="B5" s="40" t="inlineStr">
+        <is>
+          <t>מתנות</t>
+        </is>
+      </c>
+      <c r="C5" s="39" t="inlineStr">
+        <is>
+          <t>פרחים לבת זוג</t>
+        </is>
+      </c>
+      <c r="D5" s="41" t="n">
+        <v>140</v>
+      </c>
+      <c r="E5" s="39" t="inlineStr">
+        <is>
+          <t>לא צוין</t>
+        </is>
+      </c>
+      <c r="F5" s="42" t="inlineStr">
+        <is>
+          <t>❌ לא</t>
+        </is>
+      </c>
+      <c r="G5" s="39" t="inlineStr"/>
       <c r="H5" s="2" t="n"/>
       <c r="I5" s="2" t="n"/>
       <c r="J5" s="2" t="n"/>
       <c r="K5" s="2" t="n"/>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="n"/>
-      <c r="B6" s="2" t="n"/>
-      <c r="C6" s="2" t="n"/>
-      <c r="D6" s="2" t="n"/>
-      <c r="E6" s="2" t="n"/>
-      <c r="F6" s="2" t="n"/>
-      <c r="G6" s="2" t="n"/>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="43" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="B6" s="44" t="inlineStr">
+        <is>
+          <t>חשבונות קבועים</t>
+        </is>
+      </c>
+      <c r="C6" s="43" t="inlineStr">
+        <is>
+          <t>מנוי גוגל</t>
+        </is>
+      </c>
+      <c r="D6" s="45" t="n">
+        <v>8</v>
+      </c>
+      <c r="E6" s="43" t="inlineStr">
+        <is>
+          <t>כרטיס אשראי</t>
+        </is>
+      </c>
+      <c r="F6" s="47" t="inlineStr">
+        <is>
+          <t>✅ כן</t>
+        </is>
+      </c>
+      <c r="G6" s="43" t="inlineStr"/>
       <c r="H6" s="2" t="n"/>
       <c r="I6" s="2" t="n"/>
       <c r="J6" s="2" t="n"/>
       <c r="K6" s="2" t="n"/>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="n"/>
-      <c r="B7" s="2" t="n"/>
-      <c r="C7" s="2" t="n"/>
-      <c r="D7" s="2" t="n"/>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="2" t="n"/>
-      <c r="G7" s="2" t="n"/>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="39" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="B7" s="40" t="inlineStr">
+        <is>
+          <t>אחר</t>
+        </is>
+      </c>
+      <c r="C7" s="39" t="inlineStr">
+        <is>
+          <t>ביט - העברה</t>
+        </is>
+      </c>
+      <c r="D7" s="41" t="n">
+        <v>20</v>
+      </c>
+      <c r="E7" s="39" t="inlineStr">
+        <is>
+          <t>ביט</t>
+        </is>
+      </c>
+      <c r="F7" s="42" t="inlineStr">
+        <is>
+          <t>❌ לא</t>
+        </is>
+      </c>
+      <c r="G7" s="39" t="inlineStr">
+        <is>
+          <t>לא ידוע למה</t>
+        </is>
+      </c>
       <c r="H7" s="2" t="n"/>
       <c r="I7" s="2" t="n"/>
       <c r="J7" s="2" t="n"/>
       <c r="K7" s="2" t="n"/>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="n"/>
-      <c r="B8" s="2" t="n"/>
-      <c r="C8" s="2" t="n"/>
-      <c r="D8" s="2" t="n"/>
-      <c r="E8" s="2" t="n"/>
-      <c r="F8" s="2" t="n"/>
-      <c r="G8" s="2" t="n"/>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="43" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="B8" s="44" t="inlineStr">
+        <is>
+          <t>מסעדות וקפה</t>
+        </is>
+      </c>
+      <c r="C8" s="43" t="inlineStr">
+        <is>
+          <t>משלוח אוכל</t>
+        </is>
+      </c>
+      <c r="D8" s="45" t="n">
+        <v>118</v>
+      </c>
+      <c r="E8" s="43" t="inlineStr">
+        <is>
+          <t>לא צוין</t>
+        </is>
+      </c>
+      <c r="F8" s="46" t="inlineStr">
+        <is>
+          <t>❌ לא</t>
+        </is>
+      </c>
+      <c r="G8" s="43" t="inlineStr"/>
       <c r="H8" s="2" t="n"/>
       <c r="I8" s="2" t="n"/>
       <c r="J8" s="2" t="n"/>
       <c r="K8" s="2" t="n"/>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="n"/>
-      <c r="B9" s="2" t="n"/>
-      <c r="C9" s="2" t="n"/>
-      <c r="D9" s="2" t="n"/>
-      <c r="E9" s="2" t="n"/>
-      <c r="F9" s="2" t="n"/>
-      <c r="G9" s="2" t="n"/>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="39" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="B9" s="40" t="inlineStr">
+        <is>
+          <t>מזון וסופר</t>
+        </is>
+      </c>
+      <c r="C9" s="39" t="inlineStr">
+        <is>
+          <t>שופרסל</t>
+        </is>
+      </c>
+      <c r="D9" s="41" t="n">
+        <v>64</v>
+      </c>
+      <c r="E9" s="39" t="inlineStr">
+        <is>
+          <t>לא צוין</t>
+        </is>
+      </c>
+      <c r="F9" s="48" t="inlineStr">
+        <is>
+          <t>✅ כן</t>
+        </is>
+      </c>
+      <c r="G9" s="39" t="inlineStr"/>
       <c r="H9" s="2" t="n"/>
       <c r="I9" s="2" t="n"/>
       <c r="J9" s="2" t="n"/>
       <c r="K9" s="2" t="n"/>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="n"/>
-      <c r="B10" s="2" t="n"/>
-      <c r="C10" s="2" t="n"/>
-      <c r="D10" s="2" t="n"/>
-      <c r="E10" s="2" t="n"/>
-      <c r="F10" s="2" t="n"/>
-      <c r="G10" s="2" t="n"/>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="43" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="B10" s="44" t="inlineStr">
+        <is>
+          <t>מסעדות וקפה</t>
+        </is>
+      </c>
+      <c r="C10" s="43" t="inlineStr">
+        <is>
+          <t>פסאו - מסעדה</t>
+        </is>
+      </c>
+      <c r="D10" s="45" t="n">
+        <v>286</v>
+      </c>
+      <c r="E10" s="43" t="inlineStr">
+        <is>
+          <t>לא צוין</t>
+        </is>
+      </c>
+      <c r="F10" s="46" t="inlineStr">
+        <is>
+          <t>❌ לא</t>
+        </is>
+      </c>
+      <c r="G10" s="43" t="inlineStr"/>
       <c r="H10" s="2" t="n"/>
       <c r="I10" s="2" t="n"/>
       <c r="J10" s="2" t="n"/>
       <c r="K10" s="2" t="n"/>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="n"/>
-      <c r="B11" s="2" t="n"/>
-      <c r="C11" s="2" t="n"/>
-      <c r="D11" s="2" t="n"/>
-      <c r="E11" s="2" t="n"/>
-      <c r="F11" s="2" t="n"/>
-      <c r="G11" s="2" t="n"/>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="39" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="B11" s="40" t="inlineStr">
+        <is>
+          <t>מסעדות וקפה</t>
+        </is>
+      </c>
+      <c r="C11" s="39" t="inlineStr">
+        <is>
+          <t>פריים - מסעדה</t>
+        </is>
+      </c>
+      <c r="D11" s="41" t="n">
+        <v>120</v>
+      </c>
+      <c r="E11" s="39" t="inlineStr">
+        <is>
+          <t>לא צוין</t>
+        </is>
+      </c>
+      <c r="F11" s="42" t="inlineStr">
+        <is>
+          <t>❌ לא</t>
+        </is>
+      </c>
+      <c r="G11" s="39" t="inlineStr"/>
       <c r="H11" s="2" t="n"/>
       <c r="I11" s="2" t="n"/>
       <c r="J11" s="2" t="n"/>
       <c r="K11" s="2" t="n"/>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="n"/>
-      <c r="B12" s="2" t="n"/>
-      <c r="C12" s="2" t="n"/>
-      <c r="D12" s="2" t="n"/>
-      <c r="E12" s="2" t="n"/>
-      <c r="F12" s="2" t="n"/>
-      <c r="G12" s="2" t="n"/>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="43" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="B12" s="44" t="inlineStr">
+        <is>
+          <t>מסעדות וקפה</t>
+        </is>
+      </c>
+      <c r="C12" s="43" t="inlineStr">
+        <is>
+          <t>משלוח אוכל</t>
+        </is>
+      </c>
+      <c r="D12" s="45" t="n">
+        <v>83</v>
+      </c>
+      <c r="E12" s="43" t="inlineStr">
+        <is>
+          <t>לא צוין</t>
+        </is>
+      </c>
+      <c r="F12" s="46" t="inlineStr">
+        <is>
+          <t>❌ לא</t>
+        </is>
+      </c>
+      <c r="G12" s="43" t="inlineStr"/>
       <c r="H12" s="2" t="n"/>
       <c r="I12" s="2" t="n"/>
       <c r="J12" s="2" t="n"/>
       <c r="K12" s="2" t="n"/>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="n"/>
-      <c r="B13" s="2" t="n"/>
-      <c r="C13" s="2" t="n"/>
-      <c r="D13" s="2" t="n"/>
-      <c r="E13" s="2" t="n"/>
-      <c r="F13" s="2" t="n"/>
-      <c r="G13" s="2" t="n"/>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="39" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="B13" s="40" t="inlineStr">
+        <is>
+          <t>מסעדות וקפה</t>
+        </is>
+      </c>
+      <c r="C13" s="39" t="inlineStr">
+        <is>
+          <t>קולה</t>
+        </is>
+      </c>
+      <c r="D13" s="41" t="n">
+        <v>8</v>
+      </c>
+      <c r="E13" s="39" t="inlineStr">
+        <is>
+          <t>מזומן</t>
+        </is>
+      </c>
+      <c r="F13" s="42" t="inlineStr">
+        <is>
+          <t>❌ לא</t>
+        </is>
+      </c>
+      <c r="G13" s="39" t="inlineStr"/>
       <c r="H13" s="2" t="n"/>
       <c r="I13" s="2" t="n"/>
       <c r="J13" s="2" t="n"/>
       <c r="K13" s="2" t="n"/>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="n"/>
-      <c r="B14" s="2" t="n"/>
-      <c r="C14" s="2" t="n"/>
-      <c r="D14" s="2" t="n"/>
-      <c r="E14" s="2" t="n"/>
-      <c r="F14" s="2" t="n"/>
-      <c r="G14" s="2" t="n"/>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="43" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="B14" s="44" t="inlineStr">
+        <is>
+          <t>מסעדות וקפה</t>
+        </is>
+      </c>
+      <c r="C14" s="43" t="inlineStr">
+        <is>
+          <t>ארומה - כריך וקפה</t>
+        </is>
+      </c>
+      <c r="D14" s="45" t="n">
+        <v>15</v>
+      </c>
+      <c r="E14" s="43" t="inlineStr">
+        <is>
+          <t>לא צוין</t>
+        </is>
+      </c>
+      <c r="F14" s="46" t="inlineStr">
+        <is>
+          <t>❌ לא</t>
+        </is>
+      </c>
+      <c r="G14" s="43" t="inlineStr"/>
       <c r="H14" s="2" t="n"/>
       <c r="I14" s="2" t="n"/>
       <c r="J14" s="2" t="n"/>
       <c r="K14" s="2" t="n"/>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="n"/>
-      <c r="B15" s="2" t="n"/>
-      <c r="C15" s="2" t="n"/>
-      <c r="D15" s="2" t="n"/>
-      <c r="E15" s="2" t="n"/>
-      <c r="F15" s="2" t="n"/>
-      <c r="G15" s="2" t="n"/>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="39" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="B15" s="40" t="inlineStr">
+        <is>
+          <t>מסעדות וקפה</t>
+        </is>
+      </c>
+      <c r="C15" s="39" t="inlineStr">
+        <is>
+          <t>משקה אנרגיה</t>
+        </is>
+      </c>
+      <c r="D15" s="41" t="n">
+        <v>10</v>
+      </c>
+      <c r="E15" s="39" t="inlineStr">
+        <is>
+          <t>מזומן</t>
+        </is>
+      </c>
+      <c r="F15" s="42" t="inlineStr">
+        <is>
+          <t>❌ לא</t>
+        </is>
+      </c>
+      <c r="G15" s="39" t="inlineStr"/>
       <c r="H15" s="2" t="n"/>
       <c r="I15" s="2" t="n"/>
       <c r="J15" s="2" t="n"/>
       <c r="K15" s="2" t="n"/>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="n"/>
-      <c r="B16" s="2" t="n"/>
-      <c r="C16" s="2" t="n"/>
-      <c r="D16" s="2" t="n"/>
-      <c r="E16" s="2" t="n"/>
-      <c r="F16" s="2" t="n"/>
-      <c r="G16" s="2" t="n"/>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="43" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="B16" s="44" t="inlineStr">
+        <is>
+          <t>בילויים</t>
+        </is>
+      </c>
+      <c r="C16" s="43" t="inlineStr">
+        <is>
+          <t>באולינג ומשחקייה</t>
+        </is>
+      </c>
+      <c r="D16" s="45" t="n">
+        <v>66</v>
+      </c>
+      <c r="E16" s="43" t="inlineStr">
+        <is>
+          <t>לא צוין</t>
+        </is>
+      </c>
+      <c r="F16" s="46" t="inlineStr">
+        <is>
+          <t>❌ לא</t>
+        </is>
+      </c>
+      <c r="G16" s="43" t="inlineStr"/>
       <c r="H16" s="2" t="n"/>
       <c r="I16" s="2" t="n"/>
       <c r="J16" s="2" t="n"/>
       <c r="K16" s="2" t="n"/>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="n"/>
-      <c r="B17" s="2" t="n"/>
-      <c r="C17" s="2" t="n"/>
-      <c r="D17" s="2" t="n"/>
-      <c r="E17" s="2" t="n"/>
-      <c r="F17" s="2" t="n"/>
-      <c r="G17" s="2" t="n"/>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="39" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="B17" s="40" t="inlineStr">
+        <is>
+          <t>אחר</t>
+        </is>
+      </c>
+      <c r="C17" s="39" t="inlineStr">
+        <is>
+          <t>תרומה - חיות בכבוד</t>
+        </is>
+      </c>
+      <c r="D17" s="41" t="n">
+        <v>189</v>
+      </c>
+      <c r="E17" s="39" t="inlineStr">
+        <is>
+          <t>לא צוין</t>
+        </is>
+      </c>
+      <c r="F17" s="42" t="inlineStr">
+        <is>
+          <t>❌ לא</t>
+        </is>
+      </c>
+      <c r="G17" s="39" t="inlineStr">
+        <is>
+          <t>תרומה לעמותה</t>
+        </is>
+      </c>
       <c r="H17" s="2" t="n"/>
       <c r="I17" s="2" t="n"/>
       <c r="J17" s="2" t="n"/>
       <c r="K17" s="2" t="n"/>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="n"/>
-      <c r="B18" s="2" t="n"/>
-      <c r="C18" s="2" t="n"/>
-      <c r="D18" s="2" t="n"/>
-      <c r="E18" s="2" t="n"/>
-      <c r="F18" s="2" t="n"/>
-      <c r="G18" s="2" t="n"/>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="43" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="B18" s="44" t="inlineStr">
+        <is>
+          <t>מסעדות וקפה</t>
+        </is>
+      </c>
+      <c r="C18" s="43" t="inlineStr">
+        <is>
+          <t>עזרא ובניו - אוכל</t>
+        </is>
+      </c>
+      <c r="D18" s="45" t="n">
+        <v>65</v>
+      </c>
+      <c r="E18" s="43" t="inlineStr">
+        <is>
+          <t>לא צוין</t>
+        </is>
+      </c>
+      <c r="F18" s="46" t="inlineStr">
+        <is>
+          <t>❌ לא</t>
+        </is>
+      </c>
+      <c r="G18" s="43" t="inlineStr"/>
       <c r="H18" s="2" t="n"/>
       <c r="I18" s="2" t="n"/>
       <c r="J18" s="2" t="n"/>
       <c r="K18" s="2" t="n"/>
     </row>
-    <row r="19">
-      <c r="A19" s="2" t="n"/>
-      <c r="B19" s="2" t="n"/>
-      <c r="C19" s="2" t="n"/>
-      <c r="D19" s="2" t="n"/>
-      <c r="E19" s="2" t="n"/>
-      <c r="F19" s="2" t="n"/>
-      <c r="G19" s="2" t="n"/>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="39" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="B19" s="40" t="inlineStr">
+        <is>
+          <t>מתנות</t>
+        </is>
+      </c>
+      <c r="C19" s="39" t="inlineStr">
+        <is>
+          <t>פרחים לבת זוג</t>
+        </is>
+      </c>
+      <c r="D19" s="41" t="n">
+        <v>205</v>
+      </c>
+      <c r="E19" s="39" t="inlineStr">
+        <is>
+          <t>לא צוין</t>
+        </is>
+      </c>
+      <c r="F19" s="42" t="inlineStr">
+        <is>
+          <t>❌ לא</t>
+        </is>
+      </c>
+      <c r="G19" s="39" t="inlineStr"/>
       <c r="H19" s="2" t="n"/>
       <c r="I19" s="2" t="n"/>
       <c r="J19" s="2" t="n"/>
       <c r="K19" s="2" t="n"/>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="n"/>
-      <c r="B20" s="2" t="n"/>
-      <c r="C20" s="2" t="n"/>
-      <c r="D20" s="2" t="n"/>
-      <c r="E20" s="2" t="n"/>
-      <c r="F20" s="2" t="n"/>
-      <c r="G20" s="2" t="n"/>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="43" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="B20" s="44" t="inlineStr">
+        <is>
+          <t>מסעדות וקפה</t>
+        </is>
+      </c>
+      <c r="C20" s="43" t="inlineStr">
+        <is>
+          <t>משקה אנרגיה</t>
+        </is>
+      </c>
+      <c r="D20" s="45" t="n">
+        <v>16</v>
+      </c>
+      <c r="E20" s="43" t="inlineStr">
+        <is>
+          <t>מזומן</t>
+        </is>
+      </c>
+      <c r="F20" s="46" t="inlineStr">
+        <is>
+          <t>❌ לא</t>
+        </is>
+      </c>
+      <c r="G20" s="43" t="inlineStr"/>
       <c r="H20" s="2" t="n"/>
       <c r="I20" s="2" t="n"/>
       <c r="J20" s="2" t="n"/>
       <c r="K20" s="2" t="n"/>
     </row>
-    <row r="21">
-      <c r="A21" s="2" t="n"/>
-      <c r="B21" s="2" t="n"/>
-      <c r="C21" s="2" t="n"/>
-      <c r="D21" s="2" t="n"/>
-      <c r="E21" s="2" t="n"/>
-      <c r="F21" s="2" t="n"/>
-      <c r="G21" s="2" t="n"/>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="39" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="B21" s="40" t="inlineStr">
+        <is>
+          <t>ביגוד והנעלה</t>
+        </is>
+      </c>
+      <c r="C21" s="39" t="inlineStr">
+        <is>
+          <t>ריקושט - כומתה</t>
+        </is>
+      </c>
+      <c r="D21" s="41" t="n">
+        <v>31</v>
+      </c>
+      <c r="E21" s="39" t="inlineStr">
+        <is>
+          <t>לא צוין</t>
+        </is>
+      </c>
+      <c r="F21" s="48" t="inlineStr">
+        <is>
+          <t>✅ כן</t>
+        </is>
+      </c>
+      <c r="G21" s="39" t="inlineStr">
+        <is>
+          <t>ציוד צבאי</t>
+        </is>
+      </c>
       <c r="H21" s="2" t="n"/>
       <c r="I21" s="2" t="n"/>
       <c r="J21" s="2" t="n"/>
       <c r="K21" s="2" t="n"/>
     </row>
-    <row r="22">
-      <c r="A22" s="2" t="n"/>
-      <c r="B22" s="2" t="n"/>
-      <c r="C22" s="2" t="n"/>
-      <c r="D22" s="2" t="n"/>
-      <c r="E22" s="2" t="n"/>
-      <c r="F22" s="2" t="n"/>
-      <c r="G22" s="2" t="n"/>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="43" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="B22" s="44" t="inlineStr">
+        <is>
+          <t>מסעדות וקפה</t>
+        </is>
+      </c>
+      <c r="C22" s="43" t="inlineStr">
+        <is>
+          <t>ספייס - משקה</t>
+        </is>
+      </c>
+      <c r="D22" s="45" t="n">
+        <v>20</v>
+      </c>
+      <c r="E22" s="43" t="inlineStr">
+        <is>
+          <t>לא צוין</t>
+        </is>
+      </c>
+      <c r="F22" s="46" t="inlineStr">
+        <is>
+          <t>❌ לא</t>
+        </is>
+      </c>
+      <c r="G22" s="43" t="inlineStr"/>
       <c r="H22" s="2" t="n"/>
       <c r="I22" s="2" t="n"/>
       <c r="J22" s="2" t="n"/>
       <c r="K22" s="2" t="n"/>
     </row>
-    <row r="23">
-      <c r="A23" s="2" t="n"/>
-      <c r="B23" s="2" t="n"/>
-      <c r="C23" s="2" t="n"/>
-      <c r="D23" s="2" t="n"/>
-      <c r="E23" s="2" t="n"/>
-      <c r="F23" s="2" t="n"/>
-      <c r="G23" s="2" t="n"/>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="39" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="B23" s="40" t="inlineStr">
+        <is>
+          <t>מסעדות וקפה</t>
+        </is>
+      </c>
+      <c r="C23" s="39" t="inlineStr">
+        <is>
+          <t>גלידה לבת זוג</t>
+        </is>
+      </c>
+      <c r="D23" s="41" t="n">
+        <v>30</v>
+      </c>
+      <c r="E23" s="39" t="inlineStr">
+        <is>
+          <t>מזומן</t>
+        </is>
+      </c>
+      <c r="F23" s="42" t="inlineStr">
+        <is>
+          <t>❌ לא</t>
+        </is>
+      </c>
+      <c r="G23" s="39" t="inlineStr"/>
       <c r="H23" s="2" t="n"/>
       <c r="I23" s="2" t="n"/>
       <c r="J23" s="2" t="n"/>
       <c r="K23" s="2" t="n"/>
     </row>
-    <row r="24">
-      <c r="A24" s="2" t="n"/>
-      <c r="B24" s="2" t="n"/>
-      <c r="C24" s="2" t="n"/>
-      <c r="D24" s="2" t="n"/>
-      <c r="E24" s="2" t="n"/>
-      <c r="F24" s="2" t="n"/>
-      <c r="G24" s="2" t="n"/>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="43" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="B24" s="44" t="inlineStr">
+        <is>
+          <t>חינוך</t>
+        </is>
+      </c>
+      <c r="C24" s="43" t="inlineStr">
+        <is>
+          <t>שיעורי נהיגה</t>
+        </is>
+      </c>
+      <c r="D24" s="45" t="n">
+        <v>300</v>
+      </c>
+      <c r="E24" s="43" t="inlineStr">
+        <is>
+          <t>לא צוין</t>
+        </is>
+      </c>
+      <c r="F24" s="47" t="inlineStr">
+        <is>
+          <t>✅ כן</t>
+        </is>
+      </c>
+      <c r="G24" s="43" t="inlineStr"/>
       <c r="H24" s="2" t="n"/>
       <c r="I24" s="2" t="n"/>
       <c r="J24" s="2" t="n"/>
       <c r="K24" s="2" t="n"/>
     </row>
-    <row r="25">
-      <c r="A25" s="2" t="n"/>
-      <c r="B25" s="2" t="n"/>
-      <c r="C25" s="2" t="n"/>
-      <c r="D25" s="2" t="n"/>
-      <c r="E25" s="2" t="n"/>
-      <c r="F25" s="2" t="n"/>
-      <c r="G25" s="2" t="n"/>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="39" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="B25" s="40" t="inlineStr">
+        <is>
+          <t>אחר</t>
+        </is>
+      </c>
+      <c r="C25" s="39" t="inlineStr">
+        <is>
+          <t>KSP - 2 ראשי מטען + 2 מולטי ויטמין</t>
+        </is>
+      </c>
+      <c r="D25" s="41" t="n">
+        <v>365</v>
+      </c>
+      <c r="E25" s="39" t="inlineStr">
+        <is>
+          <t>לא צוין</t>
+        </is>
+      </c>
+      <c r="F25" s="48" t="inlineStr">
+        <is>
+          <t>✅ כן</t>
+        </is>
+      </c>
+      <c r="G25" s="39" t="inlineStr">
+        <is>
+          <t>אלקטרוניקה + ויטמינים</t>
+        </is>
+      </c>
       <c r="H25" s="2" t="n"/>
       <c r="I25" s="2" t="n"/>
       <c r="J25" s="2" t="n"/>
       <c r="K25" s="2" t="n"/>
     </row>
-    <row r="26">
-      <c r="A26" s="2" t="n"/>
-      <c r="B26" s="2" t="n"/>
-      <c r="C26" s="2" t="n"/>
-      <c r="D26" s="2" t="n"/>
-      <c r="E26" s="2" t="n"/>
-      <c r="F26" s="2" t="n"/>
-      <c r="G26" s="2" t="n"/>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="43" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="B26" s="44" t="inlineStr">
+        <is>
+          <t>מסעדות וקפה</t>
+        </is>
+      </c>
+      <c r="C26" s="43" t="inlineStr">
+        <is>
+          <t>ארומה - כריך</t>
+        </is>
+      </c>
+      <c r="D26" s="45" t="n">
+        <v>15</v>
+      </c>
+      <c r="E26" s="43" t="inlineStr">
+        <is>
+          <t>לא צוין</t>
+        </is>
+      </c>
+      <c r="F26" s="46" t="inlineStr">
+        <is>
+          <t>❌ לא</t>
+        </is>
+      </c>
+      <c r="G26" s="43" t="inlineStr"/>
       <c r="H26" s="2" t="n"/>
       <c r="I26" s="2" t="n"/>
       <c r="J26" s="2" t="n"/>
       <c r="K26" s="2" t="n"/>
     </row>
-    <row r="27">
-      <c r="A27" s="2" t="n"/>
-      <c r="B27" s="2" t="n"/>
-      <c r="C27" s="2" t="n"/>
-      <c r="D27" s="2" t="n"/>
-      <c r="E27" s="2" t="n"/>
-      <c r="F27" s="2" t="n"/>
-      <c r="G27" s="2" t="n"/>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="39" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="B27" s="40" t="inlineStr">
+        <is>
+          <t>אחר</t>
+        </is>
+      </c>
+      <c r="C27" s="39" t="inlineStr">
+        <is>
+          <t>אוזניות וכבל לטלפון</t>
+        </is>
+      </c>
+      <c r="D27" s="41" t="n">
+        <v>349</v>
+      </c>
+      <c r="E27" s="39" t="inlineStr">
+        <is>
+          <t>לא צוין</t>
+        </is>
+      </c>
+      <c r="F27" s="42" t="inlineStr">
+        <is>
+          <t>❌ לא</t>
+        </is>
+      </c>
+      <c r="G27" s="39" t="inlineStr">
+        <is>
+          <t>אלקטרוניקה</t>
+        </is>
+      </c>
       <c r="H27" s="2" t="n"/>
       <c r="I27" s="2" t="n"/>
       <c r="J27" s="2" t="n"/>
       <c r="K27" s="2" t="n"/>
     </row>
-    <row r="28">
-      <c r="A28" s="2" t="n"/>
-      <c r="B28" s="2" t="n"/>
-      <c r="C28" s="2" t="n"/>
-      <c r="D28" s="2" t="n"/>
-      <c r="E28" s="2" t="n"/>
-      <c r="F28" s="2" t="n"/>
-      <c r="G28" s="2" t="n"/>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="43" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="B28" s="44" t="inlineStr">
+        <is>
+          <t>מסעדות וקפה</t>
+        </is>
+      </c>
+      <c r="C28" s="43" t="inlineStr">
+        <is>
+          <t>משקה אנרגיה</t>
+        </is>
+      </c>
+      <c r="D28" s="45" t="n">
+        <v>11</v>
+      </c>
+      <c r="E28" s="43" t="inlineStr">
+        <is>
+          <t>מזומן</t>
+        </is>
+      </c>
+      <c r="F28" s="46" t="inlineStr">
+        <is>
+          <t>❌ לא</t>
+        </is>
+      </c>
+      <c r="G28" s="43" t="inlineStr"/>
       <c r="H28" s="2" t="n"/>
       <c r="I28" s="2" t="n"/>
       <c r="J28" s="2" t="n"/>
       <c r="K28" s="2" t="n"/>
     </row>
-    <row r="29">
-      <c r="A29" s="2" t="n"/>
-      <c r="B29" s="2" t="n"/>
-      <c r="C29" s="2" t="n"/>
-      <c r="D29" s="2" t="n"/>
-      <c r="E29" s="2" t="n"/>
-      <c r="F29" s="2" t="n"/>
-      <c r="G29" s="2" t="n"/>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="39" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="B29" s="40" t="inlineStr">
+        <is>
+          <t>מסעדות וקפה</t>
+        </is>
+      </c>
+      <c r="C29" s="39" t="inlineStr">
+        <is>
+          <t>משקה אנרגיה</t>
+        </is>
+      </c>
+      <c r="D29" s="41" t="n">
+        <v>14</v>
+      </c>
+      <c r="E29" s="39" t="inlineStr">
+        <is>
+          <t>מזומן</t>
+        </is>
+      </c>
+      <c r="F29" s="42" t="inlineStr">
+        <is>
+          <t>❌ לא</t>
+        </is>
+      </c>
+      <c r="G29" s="39" t="inlineStr"/>
       <c r="H29" s="2" t="n"/>
       <c r="I29" s="2" t="n"/>
       <c r="J29" s="2" t="n"/>
       <c r="K29" s="2" t="n"/>
     </row>
-    <row r="30">
-      <c r="A30" s="2" t="n"/>
-      <c r="B30" s="2" t="n"/>
-      <c r="C30" s="2" t="n"/>
-      <c r="D30" s="2" t="n"/>
-      <c r="E30" s="2" t="n"/>
-      <c r="F30" s="2" t="n"/>
-      <c r="G30" s="2" t="n"/>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="43" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="B30" s="44" t="inlineStr">
+        <is>
+          <t>מזון וסופר</t>
+        </is>
+      </c>
+      <c r="C30" s="43" t="inlineStr">
+        <is>
+          <t>קניות סופר + מברשת שיניים חשמלית</t>
+        </is>
+      </c>
+      <c r="D30" s="45" t="n">
+        <v>304</v>
+      </c>
+      <c r="E30" s="43" t="inlineStr">
+        <is>
+          <t>לא צוין</t>
+        </is>
+      </c>
+      <c r="F30" s="47" t="inlineStr">
+        <is>
+          <t>✅ כן</t>
+        </is>
+      </c>
+      <c r="G30" s="43" t="inlineStr"/>
       <c r="H30" s="2" t="n"/>
       <c r="I30" s="2" t="n"/>
       <c r="J30" s="2" t="n"/>
       <c r="K30" s="2" t="n"/>
     </row>
-    <row r="31">
-      <c r="A31" s="2" t="n"/>
-      <c r="B31" s="2" t="n"/>
-      <c r="C31" s="2" t="n"/>
-      <c r="D31" s="2" t="n"/>
-      <c r="E31" s="2" t="n"/>
-      <c r="F31" s="2" t="n"/>
-      <c r="G31" s="2" t="n"/>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="39" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="B31" s="40" t="inlineStr">
+        <is>
+          <t>בריאות ורפואה</t>
+        </is>
+      </c>
+      <c r="C31" s="39" t="inlineStr">
+        <is>
+          <t>תספורת</t>
+        </is>
+      </c>
+      <c r="D31" s="41" t="n">
+        <v>120</v>
+      </c>
+      <c r="E31" s="39" t="inlineStr">
+        <is>
+          <t>מזומן</t>
+        </is>
+      </c>
+      <c r="F31" s="48" t="inlineStr">
+        <is>
+          <t>✅ כן</t>
+        </is>
+      </c>
+      <c r="G31" s="39" t="inlineStr"/>
       <c r="H31" s="2" t="n"/>
       <c r="I31" s="2" t="n"/>
       <c r="J31" s="2" t="n"/>
       <c r="K31" s="2" t="n"/>
     </row>
-    <row r="32">
-      <c r="A32" s="2" t="n"/>
-      <c r="B32" s="2" t="n"/>
-      <c r="C32" s="2" t="n"/>
-      <c r="D32" s="2" t="n"/>
-      <c r="E32" s="2" t="n"/>
-      <c r="F32" s="2" t="n"/>
-      <c r="G32" s="2" t="n"/>
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="43" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="B32" s="44" t="inlineStr">
+        <is>
+          <t>חינוך</t>
+        </is>
+      </c>
+      <c r="C32" s="43" t="inlineStr">
+        <is>
+          <t>שיעורי נהיגה - העברה בנקאית</t>
+        </is>
+      </c>
+      <c r="D32" s="45" t="n">
+        <v>800</v>
+      </c>
+      <c r="E32" s="43" t="inlineStr">
+        <is>
+          <t>העברה בנקאית</t>
+        </is>
+      </c>
+      <c r="F32" s="47" t="inlineStr">
+        <is>
+          <t>✅ כן</t>
+        </is>
+      </c>
+      <c r="G32" s="43" t="inlineStr"/>
       <c r="H32" s="2" t="n"/>
       <c r="I32" s="2" t="n"/>
       <c r="J32" s="2" t="n"/>
@@ -10277,7 +11184,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1">
-      <c r="A1" s="33" t="inlineStr">
+      <c r="A1" s="49" t="inlineStr">
         <is>
           <t>📋  הוצאות קבועות חודשיות</t>
         </is>
@@ -10285,42 +11192,42 @@
       <c r="K1" s="2" t="n"/>
     </row>
     <row r="2" ht="26" customHeight="1">
-      <c r="A2" s="34" t="inlineStr">
+      <c r="A2" s="50" t="inlineStr">
         <is>
           <t>הוצאה</t>
         </is>
       </c>
-      <c r="B2" s="34" t="inlineStr">
+      <c r="B2" s="50" t="inlineStr">
         <is>
           <t>קטגוריה</t>
         </is>
       </c>
-      <c r="C2" s="34" t="inlineStr">
+      <c r="C2" s="50" t="inlineStr">
         <is>
           <t>סכום</t>
         </is>
       </c>
-      <c r="D2" s="34" t="inlineStr">
+      <c r="D2" s="50" t="inlineStr">
         <is>
           <t>יום חיוב</t>
         </is>
       </c>
-      <c r="E2" s="34" t="inlineStr">
+      <c r="E2" s="50" t="inlineStr">
         <is>
           <t>שיטת תשלום</t>
         </is>
       </c>
-      <c r="F2" s="34" t="inlineStr">
+      <c r="F2" s="50" t="inlineStr">
         <is>
           <t>חיוני?</t>
         </is>
       </c>
-      <c r="G2" s="34" t="inlineStr">
+      <c r="G2" s="50" t="inlineStr">
         <is>
           <t>אפשרי לחסוך?</t>
         </is>
       </c>
-      <c r="H2" s="34" t="inlineStr">
+      <c r="H2" s="50" t="inlineStr">
         <is>
           <t>הערות</t>
         </is>
@@ -10330,40 +11237,40 @@
       <c r="K2" s="2" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="35" t="inlineStr">
+      <c r="A3" s="51" t="inlineStr">
         <is>
           <t>מנוי Claude AI</t>
         </is>
       </c>
-      <c r="B3" s="36" t="inlineStr">
+      <c r="B3" s="52" t="inlineStr">
         <is>
           <t>חשבונות קבועים</t>
         </is>
       </c>
-      <c r="C3" s="37" t="n">
+      <c r="C3" s="53" t="n">
         <v>88</v>
       </c>
-      <c r="D3" s="38" t="inlineStr">
+      <c r="D3" s="54" t="inlineStr">
         <is>
           <t>חודשי</t>
         </is>
       </c>
-      <c r="E3" s="38" t="inlineStr">
+      <c r="E3" s="54" t="inlineStr">
         <is>
           <t>כרטיס אשראי</t>
         </is>
       </c>
-      <c r="F3" s="38" t="inlineStr">
+      <c r="F3" s="54" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="G3" s="38" t="inlineStr">
+      <c r="G3" s="54" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H3" s="38" t="inlineStr">
+      <c r="H3" s="54" t="inlineStr">
         <is>
           <t>עוזר פיננסי + AI</t>
         </is>
@@ -10373,42 +11280,42 @@
       <c r="K3" s="2" t="n"/>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="39" t="inlineStr">
+      <c r="A4" s="55" t="inlineStr">
         <is>
           <t>מנוי ChatGPT</t>
         </is>
       </c>
-      <c r="B4" s="40" t="inlineStr">
+      <c r="B4" s="56" t="inlineStr">
         <is>
           <t>חשבונות קבועים</t>
         </is>
       </c>
-      <c r="C4" s="41" t="n">
+      <c r="C4" s="57" t="n">
         <v>71</v>
       </c>
-      <c r="D4" s="42" t="inlineStr">
+      <c r="D4" s="58" t="inlineStr">
         <is>
           <t>חודשי</t>
         </is>
       </c>
-      <c r="E4" s="42" t="inlineStr">
+      <c r="E4" s="58" t="inlineStr">
         <is>
           <t>כרטיס אשראי</t>
         </is>
       </c>
-      <c r="F4" s="42" t="inlineStr">
+      <c r="F4" s="58" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="G4" s="42" t="inlineStr">
+      <c r="G4" s="58" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="H4" s="42" t="inlineStr">
-        <is>
-          <t>בדוק האם נחוץ ביחד עם Claude</t>
+      <c r="H4" s="58" t="inlineStr">
+        <is>
+          <t>⚠️ כבר יש Claude — בדוק אם נחוץ</t>
         </is>
       </c>
       <c r="I4" s="2" t="n"/>
@@ -10416,40 +11323,40 @@
       <c r="K4" s="2" t="n"/>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="35" t="inlineStr">
+      <c r="A5" s="51" t="inlineStr">
         <is>
           <t>מנוי Spotify</t>
         </is>
       </c>
-      <c r="B5" s="36" t="inlineStr">
+      <c r="B5" s="52" t="inlineStr">
         <is>
           <t>חשבונות קבועים</t>
         </is>
       </c>
-      <c r="C5" s="37" t="n">
+      <c r="C5" s="53" t="n">
         <v>36</v>
       </c>
-      <c r="D5" s="38" t="inlineStr">
+      <c r="D5" s="54" t="inlineStr">
         <is>
           <t>חודשי</t>
         </is>
       </c>
-      <c r="E5" s="38" t="inlineStr">
+      <c r="E5" s="54" t="inlineStr">
         <is>
           <t>כרטיס אשראי</t>
         </is>
       </c>
-      <c r="F5" s="38" t="inlineStr">
+      <c r="F5" s="54" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="G5" s="38" t="inlineStr">
+      <c r="G5" s="54" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="H5" s="38" t="inlineStr">
+      <c r="H5" s="54" t="inlineStr">
         <is>
           <t>מוזיקה</t>
         </is>
@@ -10459,40 +11366,40 @@
       <c r="K5" s="2" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="39" t="inlineStr">
+      <c r="A6" s="55" t="inlineStr">
         <is>
           <t>מאמן כושר - אופק זרמטי</t>
         </is>
       </c>
-      <c r="B6" s="40" t="inlineStr">
+      <c r="B6" s="56" t="inlineStr">
         <is>
           <t>ספורט</t>
         </is>
       </c>
-      <c r="C6" s="41" t="n">
+      <c r="C6" s="57" t="n">
         <v>600</v>
       </c>
-      <c r="D6" s="42" t="inlineStr">
+      <c r="D6" s="58" t="inlineStr">
         <is>
           <t>חודשי</t>
         </is>
       </c>
-      <c r="E6" s="42" t="inlineStr">
+      <c r="E6" s="58" t="inlineStr">
         <is>
           <t>העברה בנקאית</t>
         </is>
       </c>
-      <c r="F6" s="42" t="inlineStr">
+      <c r="F6" s="58" t="inlineStr">
         <is>
           <t>❌</t>
         </is>
       </c>
-      <c r="G6" s="42" t="inlineStr">
+      <c r="G6" s="58" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="H6" s="42" t="inlineStr">
+      <c r="H6" s="58" t="inlineStr">
         <is>
           <t>אימון אישי</t>
         </is>
@@ -10502,12 +11409,12 @@
       <c r="K6" s="2" t="n"/>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="43" t="inlineStr">
+      <c r="A7" s="59" t="inlineStr">
         <is>
           <t>סה"כ הוצאות קבועות</t>
         </is>
       </c>
-      <c r="C7" s="44" t="n">
+      <c r="C7" s="60" t="n">
         <v>795</v>
       </c>
       <c r="D7" s="2" t="n"/>
@@ -11483,7 +12390,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1">
-      <c r="A1" s="45" t="inlineStr">
+      <c r="A1" s="61" t="inlineStr">
         <is>
           <t>🎯  תוכנית תקציב חודשית</t>
         </is>
@@ -11491,32 +12398,32 @@
       <c r="K1" s="2" t="n"/>
     </row>
     <row r="2" ht="26" customHeight="1">
-      <c r="A2" s="46" t="inlineStr">
+      <c r="A2" s="62" t="inlineStr">
         <is>
           <t>קטגוריה</t>
         </is>
       </c>
-      <c r="B2" s="46" t="inlineStr">
+      <c r="B2" s="62" t="inlineStr">
         <is>
           <t>תקציב מתוכנן</t>
         </is>
       </c>
-      <c r="C2" s="46" t="inlineStr">
+      <c r="C2" s="62" t="inlineStr">
         <is>
           <t>הוצאה בפועל</t>
         </is>
       </c>
-      <c r="D2" s="46" t="inlineStr">
+      <c r="D2" s="62" t="inlineStr">
         <is>
           <t>הפרש</t>
         </is>
       </c>
-      <c r="E2" s="46" t="inlineStr">
+      <c r="E2" s="62" t="inlineStr">
         <is>
           <t>% ניצול</t>
         </is>
       </c>
-      <c r="F2" s="46" t="inlineStr">
+      <c r="F2" s="62" t="inlineStr">
         <is>
           <t>סטטוס</t>
         </is>
@@ -11528,26 +12435,26 @@
       <c r="K2" s="2" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="47" t="inlineStr">
+      <c r="A3" s="63" t="inlineStr">
         <is>
           <t>🛒 מזון וסופר</t>
         </is>
       </c>
-      <c r="B3" s="48" t="n">
+      <c r="B3" s="64" t="n">
         <v>350</v>
       </c>
-      <c r="C3" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" s="50" t="n">
-        <v>350</v>
-      </c>
-      <c r="E3" s="51" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" s="52" t="inlineStr">
-        <is>
-          <t>✅ בתקציב</t>
+      <c r="C3" s="65" t="n">
+        <v>368</v>
+      </c>
+      <c r="D3" s="66" t="n">
+        <v>-18</v>
+      </c>
+      <c r="E3" s="67" t="n">
+        <v>1.051428571428571</v>
+      </c>
+      <c r="F3" s="28" t="inlineStr">
+        <is>
+          <t>⚠️ קרוב לגבול</t>
         </is>
       </c>
       <c r="G3" s="2" t="n"/>
@@ -11557,26 +12464,26 @@
       <c r="K3" s="2" t="n"/>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="53" t="inlineStr">
+      <c r="A4" s="68" t="inlineStr">
         <is>
           <t>☕ מסעדות וקפה</t>
         </is>
       </c>
-      <c r="B4" s="54" t="n">
+      <c r="B4" s="69" t="n">
         <v>200</v>
       </c>
-      <c r="C4" s="55" t="n">
-        <v>0</v>
-      </c>
-      <c r="D4" s="56" t="n">
-        <v>200</v>
-      </c>
-      <c r="E4" s="57" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="52" t="inlineStr">
-        <is>
-          <t>✅ בתקציב</t>
+      <c r="C4" s="70" t="n">
+        <v>811</v>
+      </c>
+      <c r="D4" s="71" t="n">
+        <v>-611</v>
+      </c>
+      <c r="E4" s="72" t="n">
+        <v>4.055</v>
+      </c>
+      <c r="F4" s="73" t="inlineStr">
+        <is>
+          <t>🔴 חרג!</t>
         </is>
       </c>
       <c r="G4" s="2" t="n"/>
@@ -11586,24 +12493,24 @@
       <c r="K4" s="2" t="n"/>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="47" t="inlineStr">
+      <c r="A5" s="63" t="inlineStr">
         <is>
           <t>🚗 תחבורה</t>
         </is>
       </c>
-      <c r="B5" s="48" t="n">
+      <c r="B5" s="64" t="n">
         <v>150</v>
       </c>
-      <c r="C5" s="49" t="n">
+      <c r="C5" s="74" t="n">
         <v>0</v>
       </c>
-      <c r="D5" s="50" t="n">
+      <c r="D5" s="75" t="n">
         <v>150</v>
       </c>
-      <c r="E5" s="51" t="n">
+      <c r="E5" s="67" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="52" t="inlineStr">
+      <c r="F5" s="76" t="inlineStr">
         <is>
           <t>✅ בתקציב</t>
         </is>
@@ -11615,24 +12522,24 @@
       <c r="K5" s="2" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="53" t="inlineStr">
+      <c r="A6" s="68" t="inlineStr">
         <is>
           <t>🎮 בילויים</t>
         </is>
       </c>
-      <c r="B6" s="54" t="n">
+      <c r="B6" s="69" t="n">
         <v>150</v>
       </c>
-      <c r="C6" s="55" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" s="56" t="n">
-        <v>150</v>
-      </c>
-      <c r="E6" s="57" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="52" t="inlineStr">
+      <c r="C6" s="77" t="n">
+        <v>66</v>
+      </c>
+      <c r="D6" s="78" t="n">
+        <v>84</v>
+      </c>
+      <c r="E6" s="72" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="F6" s="76" t="inlineStr">
         <is>
           <t>✅ בתקציב</t>
         </is>
@@ -11644,26 +12551,26 @@
       <c r="K6" s="2" t="n"/>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="47" t="inlineStr">
+      <c r="A7" s="63" t="inlineStr">
         <is>
           <t>🏥 בריאות ורפואה</t>
         </is>
       </c>
-      <c r="B7" s="48" t="n">
+      <c r="B7" s="64" t="n">
         <v>80</v>
       </c>
-      <c r="C7" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" s="50" t="n">
-        <v>80</v>
-      </c>
-      <c r="E7" s="51" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="52" t="inlineStr">
-        <is>
-          <t>✅ בתקציב</t>
+      <c r="C7" s="65" t="n">
+        <v>120</v>
+      </c>
+      <c r="D7" s="66" t="n">
+        <v>-40</v>
+      </c>
+      <c r="E7" s="67" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F7" s="73" t="inlineStr">
+        <is>
+          <t>🔴 חרג!</t>
         </is>
       </c>
       <c r="G7" s="2" t="n"/>
@@ -11673,24 +12580,24 @@
       <c r="K7" s="2" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="53" t="inlineStr">
+      <c r="A8" s="68" t="inlineStr">
         <is>
           <t>👕 ביגוד והנעלה</t>
         </is>
       </c>
-      <c r="B8" s="54" t="n">
+      <c r="B8" s="69" t="n">
         <v>100</v>
       </c>
-      <c r="C8" s="55" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" s="56" t="n">
-        <v>100</v>
-      </c>
-      <c r="E8" s="57" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="52" t="inlineStr">
+      <c r="C8" s="77" t="n">
+        <v>31</v>
+      </c>
+      <c r="D8" s="78" t="n">
+        <v>69</v>
+      </c>
+      <c r="E8" s="72" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="F8" s="76" t="inlineStr">
         <is>
           <t>✅ בתקציב</t>
         </is>
@@ -11702,26 +12609,26 @@
       <c r="K8" s="2" t="n"/>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="47" t="inlineStr">
+      <c r="A9" s="63" t="inlineStr">
         <is>
           <t>📋 חשבונות קבועים</t>
         </is>
       </c>
-      <c r="B9" s="48" t="n">
-        <v>195</v>
-      </c>
-      <c r="C9" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="50" t="n">
-        <v>195</v>
-      </c>
-      <c r="E9" s="51" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="52" t="inlineStr">
-        <is>
-          <t>✅ בתקציב</t>
+      <c r="B9" s="64" t="n">
+        <v>200</v>
+      </c>
+      <c r="C9" s="65" t="n">
+        <v>203</v>
+      </c>
+      <c r="D9" s="66" t="n">
+        <v>-3</v>
+      </c>
+      <c r="E9" s="67" t="n">
+        <v>1.015</v>
+      </c>
+      <c r="F9" s="28" t="inlineStr">
+        <is>
+          <t>⚠️ קרוב לגבול</t>
         </is>
       </c>
       <c r="G9" s="2" t="n"/>
@@ -11731,24 +12638,24 @@
       <c r="K9" s="2" t="n"/>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="53" t="inlineStr">
+      <c r="A10" s="68" t="inlineStr">
         <is>
           <t>🏠 שכר דירה</t>
         </is>
       </c>
-      <c r="B10" s="54" t="n">
+      <c r="B10" s="69" t="n">
         <v>0</v>
       </c>
-      <c r="C10" s="55" t="n">
+      <c r="C10" s="77" t="n">
         <v>0</v>
       </c>
-      <c r="D10" s="56" t="n">
+      <c r="D10" s="78" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="57" t="n">
+      <c r="E10" s="72" t="n">
         <v>0</v>
       </c>
-      <c r="F10" s="52" t="inlineStr">
+      <c r="F10" s="76" t="inlineStr">
         <is>
           <t>✅ בתקציב</t>
         </is>
@@ -11760,26 +12667,26 @@
       <c r="K10" s="2" t="n"/>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="47" t="inlineStr">
+      <c r="A11" s="63" t="inlineStr">
         <is>
           <t>📚 חינוך</t>
         </is>
       </c>
-      <c r="B11" s="48" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="50" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="51" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="52" t="inlineStr">
-        <is>
-          <t>✅ בתקציב</t>
+      <c r="B11" s="64" t="n">
+        <v>300</v>
+      </c>
+      <c r="C11" s="65" t="n">
+        <v>1100</v>
+      </c>
+      <c r="D11" s="66" t="n">
+        <v>-800</v>
+      </c>
+      <c r="E11" s="67" t="n">
+        <v>3.666666666666667</v>
+      </c>
+      <c r="F11" s="73" t="inlineStr">
+        <is>
+          <t>🔴 חרג!</t>
         </is>
       </c>
       <c r="G11" s="2" t="n"/>
@@ -11789,24 +12696,24 @@
       <c r="K11" s="2" t="n"/>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="53" t="inlineStr">
+      <c r="A12" s="68" t="inlineStr">
         <is>
           <t>💪 ספורט</t>
         </is>
       </c>
-      <c r="B12" s="54" t="n">
+      <c r="B12" s="69" t="n">
         <v>600</v>
       </c>
-      <c r="C12" s="55" t="n">
+      <c r="C12" s="77" t="n">
+        <v>600</v>
+      </c>
+      <c r="D12" s="78" t="n">
         <v>0</v>
       </c>
-      <c r="D12" s="56" t="n">
-        <v>600</v>
-      </c>
-      <c r="E12" s="57" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="52" t="inlineStr">
+      <c r="E12" s="72" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="76" t="inlineStr">
         <is>
           <t>✅ בתקציב</t>
         </is>
@@ -11818,26 +12725,26 @@
       <c r="K12" s="2" t="n"/>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="47" t="inlineStr">
+      <c r="A13" s="63" t="inlineStr">
         <is>
           <t>🎁 מתנות</t>
         </is>
       </c>
-      <c r="B13" s="48" t="n">
-        <v>50</v>
-      </c>
-      <c r="C13" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="50" t="n">
-        <v>50</v>
-      </c>
-      <c r="E13" s="51" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="52" t="inlineStr">
-        <is>
-          <t>✅ בתקציב</t>
+      <c r="B13" s="64" t="n">
+        <v>200</v>
+      </c>
+      <c r="C13" s="65" t="n">
+        <v>860</v>
+      </c>
+      <c r="D13" s="66" t="n">
+        <v>-660</v>
+      </c>
+      <c r="E13" s="67" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="F13" s="73" t="inlineStr">
+        <is>
+          <t>🔴 חרג!</t>
         </is>
       </c>
       <c r="G13" s="2" t="n"/>
@@ -11847,24 +12754,24 @@
       <c r="K13" s="2" t="n"/>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="53" t="inlineStr">
+      <c r="A14" s="68" t="inlineStr">
         <is>
           <t>💰 חיסכון</t>
         </is>
       </c>
-      <c r="B14" s="54" t="n">
+      <c r="B14" s="69" t="n">
         <v>1000</v>
       </c>
-      <c r="C14" s="55" t="n">
+      <c r="C14" s="77" t="n">
         <v>0</v>
       </c>
-      <c r="D14" s="56" t="n">
+      <c r="D14" s="78" t="n">
         <v>1000</v>
       </c>
-      <c r="E14" s="57" t="n">
+      <c r="E14" s="72" t="n">
         <v>0</v>
       </c>
-      <c r="F14" s="52" t="inlineStr">
+      <c r="F14" s="76" t="inlineStr">
         <is>
           <t>✅ בתקציב</t>
         </is>
@@ -11876,24 +12783,24 @@
       <c r="K14" s="2" t="n"/>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="47" t="inlineStr">
+      <c r="A15" s="63" t="inlineStr">
         <is>
           <t>📈 השקעות</t>
         </is>
       </c>
-      <c r="B15" s="48" t="n">
+      <c r="B15" s="64" t="n">
         <v>0</v>
       </c>
-      <c r="C15" s="49" t="n">
+      <c r="C15" s="74" t="n">
         <v>0</v>
       </c>
-      <c r="D15" s="50" t="n">
+      <c r="D15" s="75" t="n">
         <v>0</v>
       </c>
-      <c r="E15" s="51" t="n">
+      <c r="E15" s="67" t="n">
         <v>0</v>
       </c>
-      <c r="F15" s="52" t="inlineStr">
+      <c r="F15" s="76" t="inlineStr">
         <is>
           <t>✅ בתקציב</t>
         </is>
@@ -11905,26 +12812,26 @@
       <c r="K15" s="2" t="n"/>
     </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="53" t="inlineStr">
+      <c r="A16" s="68" t="inlineStr">
         <is>
           <t>💳 אחר</t>
         </is>
       </c>
-      <c r="B16" s="54" t="n">
-        <v>100</v>
-      </c>
-      <c r="C16" s="55" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" s="56" t="n">
-        <v>100</v>
-      </c>
-      <c r="E16" s="57" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="52" t="inlineStr">
-        <is>
-          <t>✅ בתקציב</t>
+      <c r="B16" s="69" t="n">
+        <v>150</v>
+      </c>
+      <c r="C16" s="70" t="n">
+        <v>923</v>
+      </c>
+      <c r="D16" s="71" t="n">
+        <v>-773</v>
+      </c>
+      <c r="E16" s="72" t="n">
+        <v>6.153333333333333</v>
+      </c>
+      <c r="F16" s="73" t="inlineStr">
+        <is>
+          <t>🔴 חרג!</t>
         </is>
       </c>
       <c r="G16" s="2" t="n"/>
@@ -12779,39 +13686,39 @@
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1">
-      <c r="A1" s="58" t="inlineStr">
+      <c r="A1" s="79" t="inlineStr">
         <is>
           <t>📈  ניתוח הוצאות לפי קטגוריות</t>
         </is>
       </c>
     </row>
     <row r="2" ht="26" customHeight="1">
-      <c r="A2" s="59" t="inlineStr">
+      <c r="A2" s="80" t="inlineStr">
         <is>
           <t>קטגוריה</t>
         </is>
       </c>
-      <c r="B2" s="59" t="inlineStr">
+      <c r="B2" s="80" t="inlineStr">
         <is>
           <t>סה"כ החודש</t>
         </is>
       </c>
-      <c r="C2" s="59" t="inlineStr">
+      <c r="C2" s="80" t="inlineStr">
         <is>
           <t>% מסה"כ</t>
         </is>
       </c>
-      <c r="D2" s="59" t="inlineStr">
+      <c r="D2" s="80" t="inlineStr">
         <is>
           <t>ממוצע יומי</t>
         </is>
       </c>
-      <c r="E2" s="59" t="inlineStr">
+      <c r="E2" s="80" t="inlineStr">
         <is>
           <t>מספר עסקאות</t>
         </is>
       </c>
-      <c r="F2" s="59" t="inlineStr">
+      <c r="F2" s="80" t="inlineStr">
         <is>
           <t>הכי גבוה</t>
         </is>
@@ -12825,21 +13732,27 @@
       <c r="M2" s="2" t="n"/>
       <c r="N2" s="2" t="n"/>
     </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="60" t="inlineStr">
-        <is>
-          <t>סה"כ</t>
-        </is>
-      </c>
-      <c r="B3" s="61" t="n">
-        <v>0</v>
-      </c>
-      <c r="C3" s="62" t="n">
-        <v>1</v>
-      </c>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n"/>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="81" t="inlineStr">
+        <is>
+          <t>🎁 מתנות</t>
+        </is>
+      </c>
+      <c r="B3" s="82" t="n">
+        <v>860</v>
+      </c>
+      <c r="C3" s="83" t="n">
+        <v>0.1692247146792601</v>
+      </c>
+      <c r="D3" s="84" t="n">
+        <v>47.77777777777778</v>
+      </c>
+      <c r="E3" s="85" t="n">
+        <v>4</v>
+      </c>
+      <c r="F3" s="86" t="n">
+        <v>415</v>
+      </c>
       <c r="G3" s="2" t="n"/>
       <c r="H3" s="2" t="n"/>
       <c r="I3" s="2" t="n"/>
@@ -12849,13 +13762,27 @@
       <c r="M3" s="2" t="n"/>
       <c r="N3" s="2" t="n"/>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="n"/>
-      <c r="B4" s="2" t="n"/>
-      <c r="C4" s="2" t="n"/>
-      <c r="D4" s="2" t="n"/>
-      <c r="E4" s="2" t="n"/>
-      <c r="F4" s="2" t="n"/>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="87" t="inlineStr">
+        <is>
+          <t>☕ מסעדות וקפה</t>
+        </is>
+      </c>
+      <c r="B4" s="88" t="n">
+        <v>811</v>
+      </c>
+      <c r="C4" s="89" t="n">
+        <v>0.1595828414010232</v>
+      </c>
+      <c r="D4" s="90" t="n">
+        <v>45.05555555555556</v>
+      </c>
+      <c r="E4" s="91" t="n">
+        <v>14</v>
+      </c>
+      <c r="F4" s="92" t="n">
+        <v>286</v>
+      </c>
       <c r="G4" s="2" t="n"/>
       <c r="H4" s="2" t="n"/>
       <c r="I4" s="2" t="n"/>
@@ -12865,13 +13792,27 @@
       <c r="M4" s="2" t="n"/>
       <c r="N4" s="2" t="n"/>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="n"/>
-      <c r="B5" s="2" t="n"/>
-      <c r="C5" s="2" t="n"/>
-      <c r="D5" s="2" t="n"/>
-      <c r="E5" s="2" t="n"/>
-      <c r="F5" s="2" t="n"/>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="81" t="inlineStr">
+        <is>
+          <t>🛒 מזון וסופר</t>
+        </is>
+      </c>
+      <c r="B5" s="93" t="n">
+        <v>368</v>
+      </c>
+      <c r="C5" s="83" t="n">
+        <v>0.07241243604879968</v>
+      </c>
+      <c r="D5" s="84" t="n">
+        <v>20.44444444444444</v>
+      </c>
+      <c r="E5" s="85" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" s="86" t="n">
+        <v>304</v>
+      </c>
       <c r="G5" s="2" t="n"/>
       <c r="H5" s="2" t="n"/>
       <c r="I5" s="2" t="n"/>
@@ -12881,13 +13822,27 @@
       <c r="M5" s="2" t="n"/>
       <c r="N5" s="2" t="n"/>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="n"/>
-      <c r="B6" s="2" t="n"/>
-      <c r="C6" s="2" t="n"/>
-      <c r="D6" s="2" t="n"/>
-      <c r="E6" s="2" t="n"/>
-      <c r="F6" s="2" t="n"/>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="87" t="inlineStr">
+        <is>
+          <t>📋 חשבונות קבועים</t>
+        </is>
+      </c>
+      <c r="B6" s="94" t="n">
+        <v>203</v>
+      </c>
+      <c r="C6" s="89" t="n">
+        <v>0.03994490358126722</v>
+      </c>
+      <c r="D6" s="90" t="n">
+        <v>11.27777777777778</v>
+      </c>
+      <c r="E6" s="91" t="n">
+        <v>4</v>
+      </c>
+      <c r="F6" s="92" t="n">
+        <v>88</v>
+      </c>
       <c r="G6" s="2" t="n"/>
       <c r="H6" s="2" t="n"/>
       <c r="I6" s="2" t="n"/>
@@ -12897,13 +13852,27 @@
       <c r="M6" s="2" t="n"/>
       <c r="N6" s="2" t="n"/>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="n"/>
-      <c r="B7" s="2" t="n"/>
-      <c r="C7" s="2" t="n"/>
-      <c r="D7" s="2" t="n"/>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="2" t="n"/>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="81" t="inlineStr">
+        <is>
+          <t>🎮 בילויים</t>
+        </is>
+      </c>
+      <c r="B7" s="95" t="n">
+        <v>66</v>
+      </c>
+      <c r="C7" s="83" t="n">
+        <v>0.01298701298701299</v>
+      </c>
+      <c r="D7" s="84" t="n">
+        <v>3.666666666666667</v>
+      </c>
+      <c r="E7" s="85" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="86" t="n">
+        <v>66</v>
+      </c>
       <c r="G7" s="2" t="n"/>
       <c r="H7" s="2" t="n"/>
       <c r="I7" s="2" t="n"/>
@@ -12913,13 +13882,27 @@
       <c r="M7" s="2" t="n"/>
       <c r="N7" s="2" t="n"/>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="n"/>
-      <c r="B8" s="2" t="n"/>
-      <c r="C8" s="2" t="n"/>
-      <c r="D8" s="2" t="n"/>
-      <c r="E8" s="2" t="n"/>
-      <c r="F8" s="2" t="n"/>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="87" t="inlineStr">
+        <is>
+          <t>💳 אחר</t>
+        </is>
+      </c>
+      <c r="B8" s="96" t="n">
+        <v>923</v>
+      </c>
+      <c r="C8" s="89" t="n">
+        <v>0.1816214088941362</v>
+      </c>
+      <c r="D8" s="90" t="n">
+        <v>51.27777777777778</v>
+      </c>
+      <c r="E8" s="91" t="n">
+        <v>4</v>
+      </c>
+      <c r="F8" s="92" t="n">
+        <v>365</v>
+      </c>
       <c r="G8" s="2" t="n"/>
       <c r="H8" s="2" t="n"/>
       <c r="I8" s="2" t="n"/>
@@ -12929,13 +13912,27 @@
       <c r="M8" s="2" t="n"/>
       <c r="N8" s="2" t="n"/>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="n"/>
-      <c r="B9" s="2" t="n"/>
-      <c r="C9" s="2" t="n"/>
-      <c r="D9" s="2" t="n"/>
-      <c r="E9" s="2" t="n"/>
-      <c r="F9" s="2" t="n"/>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="81" t="inlineStr">
+        <is>
+          <t>👕 ביגוד והנעלה</t>
+        </is>
+      </c>
+      <c r="B9" s="97" t="n">
+        <v>31</v>
+      </c>
+      <c r="C9" s="83" t="n">
+        <v>0.006099960645415191</v>
+      </c>
+      <c r="D9" s="84" t="n">
+        <v>1.722222222222222</v>
+      </c>
+      <c r="E9" s="85" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="86" t="n">
+        <v>31</v>
+      </c>
       <c r="G9" s="2" t="n"/>
       <c r="H9" s="2" t="n"/>
       <c r="I9" s="2" t="n"/>
@@ -12945,13 +13942,27 @@
       <c r="M9" s="2" t="n"/>
       <c r="N9" s="2" t="n"/>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="n"/>
-      <c r="B10" s="2" t="n"/>
-      <c r="C10" s="2" t="n"/>
-      <c r="D10" s="2" t="n"/>
-      <c r="E10" s="2" t="n"/>
-      <c r="F10" s="2" t="n"/>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="87" t="inlineStr">
+        <is>
+          <t>🏥 בריאות ורפואה</t>
+        </is>
+      </c>
+      <c r="B10" s="98" t="n">
+        <v>120</v>
+      </c>
+      <c r="C10" s="89" t="n">
+        <v>0.02361275088547816</v>
+      </c>
+      <c r="D10" s="90" t="n">
+        <v>6.666666666666667</v>
+      </c>
+      <c r="E10" s="91" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="92" t="n">
+        <v>120</v>
+      </c>
       <c r="G10" s="2" t="n"/>
       <c r="H10" s="2" t="n"/>
       <c r="I10" s="2" t="n"/>
@@ -12961,13 +13972,27 @@
       <c r="M10" s="2" t="n"/>
       <c r="N10" s="2" t="n"/>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="n"/>
-      <c r="B11" s="2" t="n"/>
-      <c r="C11" s="2" t="n"/>
-      <c r="D11" s="2" t="n"/>
-      <c r="E11" s="2" t="n"/>
-      <c r="F11" s="2" t="n"/>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="81" t="inlineStr">
+        <is>
+          <t>📚 חינוך</t>
+        </is>
+      </c>
+      <c r="B11" s="82" t="n">
+        <v>1100</v>
+      </c>
+      <c r="C11" s="83" t="n">
+        <v>0.2164502164502164</v>
+      </c>
+      <c r="D11" s="84" t="n">
+        <v>61.11111111111111</v>
+      </c>
+      <c r="E11" s="85" t="n">
+        <v>2</v>
+      </c>
+      <c r="F11" s="86" t="n">
+        <v>800</v>
+      </c>
       <c r="G11" s="2" t="n"/>
       <c r="H11" s="2" t="n"/>
       <c r="I11" s="2" t="n"/>
@@ -12977,13 +14002,27 @@
       <c r="M11" s="2" t="n"/>
       <c r="N11" s="2" t="n"/>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="n"/>
-      <c r="B12" s="2" t="n"/>
-      <c r="C12" s="2" t="n"/>
-      <c r="D12" s="2" t="n"/>
-      <c r="E12" s="2" t="n"/>
-      <c r="F12" s="2" t="n"/>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="87" t="inlineStr">
+        <is>
+          <t>💪 ספורט</t>
+        </is>
+      </c>
+      <c r="B12" s="88" t="n">
+        <v>600</v>
+      </c>
+      <c r="C12" s="89" t="n">
+        <v>0.1180637544273908</v>
+      </c>
+      <c r="D12" s="90" t="n">
+        <v>33.33333333333334</v>
+      </c>
+      <c r="E12" s="91" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="92" t="n">
+        <v>600</v>
+      </c>
       <c r="G12" s="2" t="n"/>
       <c r="H12" s="2" t="n"/>
       <c r="I12" s="2" t="n"/>
@@ -12993,10 +14032,18 @@
       <c r="M12" s="2" t="n"/>
       <c r="N12" s="2" t="n"/>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="n"/>
-      <c r="B13" s="2" t="n"/>
-      <c r="C13" s="2" t="n"/>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="99" t="inlineStr">
+        <is>
+          <t>סה"כ</t>
+        </is>
+      </c>
+      <c r="B13" s="100" t="n">
+        <v>5082</v>
+      </c>
+      <c r="C13" s="101" t="n">
+        <v>1</v>
+      </c>
       <c r="D13" s="2" t="n"/>
       <c r="E13" s="2" t="n"/>
       <c r="F13" s="2" t="n"/>
@@ -14067,7 +15114,7 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A3"/>
+    <mergeCell ref="A13"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -14099,69 +15146,69 @@
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1">
-      <c r="A1" s="63" t="inlineStr">
+      <c r="A1" s="102" t="inlineStr">
         <is>
           <t>📄  יומן תלושי שכר</t>
         </is>
       </c>
     </row>
     <row r="2" ht="26" customHeight="1">
-      <c r="A2" s="64" t="inlineStr">
+      <c r="A2" s="103" t="inlineStr">
         <is>
           <t>חודש</t>
         </is>
       </c>
-      <c r="B2" s="64" t="inlineStr">
+      <c r="B2" s="103" t="inlineStr">
         <is>
           <t>מעסיק</t>
         </is>
       </c>
-      <c r="C2" s="64" t="inlineStr">
+      <c r="C2" s="103" t="inlineStr">
         <is>
           <t>ברוטו</t>
         </is>
       </c>
-      <c r="D2" s="64" t="inlineStr">
+      <c r="D2" s="103" t="inlineStr">
         <is>
           <t>נטו</t>
         </is>
       </c>
-      <c r="E2" s="64" t="inlineStr">
+      <c r="E2" s="103" t="inlineStr">
         <is>
           <t>מס הכנסה</t>
         </is>
       </c>
-      <c r="F2" s="64" t="inlineStr">
+      <c r="F2" s="103" t="inlineStr">
         <is>
           <t>ביטוח לאומי</t>
         </is>
       </c>
-      <c r="G2" s="64" t="inlineStr">
+      <c r="G2" s="103" t="inlineStr">
         <is>
           <t>בריאות</t>
         </is>
       </c>
-      <c r="H2" s="64" t="inlineStr">
+      <c r="H2" s="103" t="inlineStr">
         <is>
           <t>קרן פנסיה</t>
         </is>
       </c>
-      <c r="I2" s="64" t="inlineStr">
+      <c r="I2" s="103" t="inlineStr">
         <is>
           <t>קרן השתלמות</t>
         </is>
       </c>
-      <c r="J2" s="64" t="inlineStr">
+      <c r="J2" s="103" t="inlineStr">
         <is>
           <t>נסיעות</t>
         </is>
       </c>
-      <c r="K2" s="64" t="inlineStr">
+      <c r="K2" s="103" t="inlineStr">
         <is>
           <t>שעות נוספות</t>
         </is>
       </c>
-      <c r="L2" s="64" t="inlineStr">
+      <c r="L2" s="103" t="inlineStr">
         <is>
           <t>הערות</t>
         </is>

</xml_diff>

<commit_message>
Add next month planning sheet and finalize April tracker
- Added '🗓️ תכנון חודש הבא' sheet with personalized budget recommendations
- Budget advice based on April spending patterns (restaurants 811₪, gifts 860₪, etc.)
- Savings goal reminder: 1,000₪ automatic transfer on 1st of month
- Marked work salary as variable income type
- Excel now has 8 sheets total

https://claude.ai/code/session_01Cwu7SWtx13xhFUMhTaLvjR
</commit_message>
<xml_diff>
--- a/finance/מעקב_פיננסי.xlsx
+++ b/finance/מעקב_פיננסי.xlsx
@@ -14,6 +14,7 @@
     <sheet name="🎯 תקציב" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="📈 ניתוח" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="📄 תלושי שכר" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="🗓️ תכנון חודש הבא" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -27,7 +28,7 @@
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="₪#,##0.0"/>
   </numFmts>
-  <fonts count="34">
+  <fonts count="36">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -224,8 +225,19 @@
       <color rgb="0017A589"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00ECF0F1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001A1A2E"/>
+      <sz val="13"/>
+    </font>
   </fonts>
-  <fills count="24">
+  <fills count="25">
     <fill>
       <patternFill/>
     </fill>
@@ -342,6 +354,11 @@
         <fgColor rgb="0017A589"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F1C40F"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -369,7 +386,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="104">
+  <cellXfs count="118">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
@@ -676,6 +693,48 @@
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="33" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="23" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="23" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="24" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
   </cellXfs>
@@ -1078,7 +1137,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>עודכן לאחרונה: 18/04/2026 06:00</t>
+          <t>עודכן לאחרונה: 18/04/2026 06:03</t>
         </is>
       </c>
       <c r="Q2" s="2" t="n"/>
@@ -2473,12 +2532,12 @@
       </c>
       <c r="E10" s="34" t="inlineStr">
         <is>
-          <t>קבוע</t>
+          <t>משתנה</t>
         </is>
       </c>
       <c r="F10" s="34" t="inlineStr">
         <is>
-          <t>משכורת עבודה</t>
+          <t>משכורת עבודה — משתנה כל חודש | אפריל: 5,616₪</t>
         </is>
       </c>
       <c r="G10" s="2" t="n"/>
@@ -16872,4 +16931,1502 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="0017A589"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L89"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="35" customHeight="1">
+      <c r="A1" s="102" t="inlineStr">
+        <is>
+          <t>🗓️  תכנון פיננסי — חודש הבא</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="8" customHeight="1">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="29" t="inlineStr">
+        <is>
+          <t>💵  הכנסות צפויות</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="30" t="inlineStr">
+        <is>
+          <t>מקור</t>
+        </is>
+      </c>
+      <c r="B4" s="30" t="inlineStr">
+        <is>
+          <t>סכום צפוי</t>
+        </is>
+      </c>
+      <c r="C4" s="30" t="inlineStr">
+        <is>
+          <t>תאריך</t>
+        </is>
+      </c>
+      <c r="D4" s="30" t="inlineStr">
+        <is>
+          <t>הערות</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="n"/>
+      <c r="H4" s="2" t="n"/>
+      <c r="I4" s="2" t="n"/>
+      <c r="J4" s="2" t="n"/>
+      <c r="K4" s="2" t="n"/>
+      <c r="L4" s="2" t="n"/>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="31" t="inlineStr">
+        <is>
+          <t>צבא</t>
+        </is>
+      </c>
+      <c r="B5" s="104" t="n">
+        <v>1462</v>
+      </c>
+      <c r="C5" s="31" t="inlineStr">
+        <is>
+          <t>1 לחודש</t>
+        </is>
+      </c>
+      <c r="D5" s="31" t="inlineStr">
+        <is>
+          <t>קבוע</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="2" t="n"/>
+      <c r="G5" s="2" t="n"/>
+      <c r="H5" s="2" t="n"/>
+      <c r="I5" s="2" t="n"/>
+      <c r="J5" s="2" t="n"/>
+      <c r="K5" s="2" t="n"/>
+      <c r="L5" s="2" t="n"/>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="34" t="inlineStr">
+        <is>
+          <t>עבודה</t>
+        </is>
+      </c>
+      <c r="B6" s="105" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="C6" s="34" t="inlineStr">
+        <is>
+          <t>10 לחודש</t>
+        </is>
+      </c>
+      <c r="D6" s="34" t="inlineStr">
+        <is>
+          <t>⚠️ משתנה — עדכן בתחילת חודש</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="n"/>
+      <c r="G6" s="2" t="n"/>
+      <c r="H6" s="2" t="n"/>
+      <c r="I6" s="2" t="n"/>
+      <c r="J6" s="2" t="n"/>
+      <c r="K6" s="2" t="n"/>
+      <c r="L6" s="2" t="n"/>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="106" t="inlineStr">
+        <is>
+          <t>סה"כ צפוי</t>
+        </is>
+      </c>
+      <c r="B7" s="106">
+        <f>B5+B6</f>
+        <v/>
+      </c>
+      <c r="C7" s="107" t="inlineStr"/>
+      <c r="D7" s="107" t="inlineStr"/>
+      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="2" t="n"/>
+      <c r="G7" s="2" t="n"/>
+      <c r="H7" s="2" t="n"/>
+      <c r="I7" s="2" t="n"/>
+      <c r="J7" s="2" t="n"/>
+      <c r="K7" s="2" t="n"/>
+      <c r="L7" s="2" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n"/>
+      <c r="B8" s="2" t="n"/>
+      <c r="C8" s="2" t="n"/>
+      <c r="D8" s="2" t="n"/>
+      <c r="E8" s="2" t="n"/>
+      <c r="F8" s="2" t="n"/>
+      <c r="G8" s="2" t="n"/>
+      <c r="H8" s="2" t="n"/>
+      <c r="I8" s="2" t="n"/>
+      <c r="J8" s="2" t="n"/>
+      <c r="K8" s="2" t="n"/>
+      <c r="L8" s="2" t="n"/>
+    </row>
+    <row r="9" ht="8" customHeight="1">
+      <c r="A9" s="2" t="n"/>
+      <c r="B9" s="2" t="n"/>
+      <c r="C9" s="2" t="n"/>
+      <c r="D9" s="2" t="n"/>
+      <c r="E9" s="2" t="n"/>
+      <c r="F9" s="2" t="n"/>
+      <c r="G9" s="2" t="n"/>
+      <c r="H9" s="2" t="n"/>
+      <c r="I9" s="2" t="n"/>
+      <c r="J9" s="2" t="n"/>
+      <c r="K9" s="2" t="n"/>
+      <c r="L9" s="2" t="n"/>
+    </row>
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="108" t="inlineStr">
+        <is>
+          <t>🎯  תקציב מתוכנן — לפי לקחים מהחודש הנוכחי</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="62" t="inlineStr">
+        <is>
+          <t>קטגוריה</t>
+        </is>
+      </c>
+      <c r="B11" s="62" t="inlineStr">
+        <is>
+          <t>הוצאה החודש</t>
+        </is>
+      </c>
+      <c r="C11" s="62" t="inlineStr">
+        <is>
+          <t>תקציב מומלץ</t>
+        </is>
+      </c>
+      <c r="D11" s="62" t="inlineStr">
+        <is>
+          <t>הפרש</t>
+        </is>
+      </c>
+      <c r="E11" s="62" t="inlineStr">
+        <is>
+          <t>הסבר</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="n"/>
+      <c r="G11" s="2" t="n"/>
+      <c r="H11" s="2" t="n"/>
+      <c r="I11" s="2" t="n"/>
+      <c r="J11" s="2" t="n"/>
+      <c r="K11" s="2" t="n"/>
+      <c r="L11" s="2" t="n"/>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="63" t="inlineStr">
+        <is>
+          <t>🛒 מזון וסופר</t>
+        </is>
+      </c>
+      <c r="B12" s="65" t="n">
+        <v>368</v>
+      </c>
+      <c r="C12" s="64" t="n">
+        <v>350</v>
+      </c>
+      <c r="D12" s="109" t="n">
+        <v>-18</v>
+      </c>
+      <c r="E12" s="110" t="inlineStr">
+        <is>
+          <t>✅ סביר — נסה להישאר מתחת ל-350₪</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="n"/>
+      <c r="G12" s="2" t="n"/>
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="2" t="n"/>
+      <c r="J12" s="2" t="n"/>
+      <c r="K12" s="2" t="n"/>
+      <c r="L12" s="2" t="n"/>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="68" t="inlineStr">
+        <is>
+          <t>☕ מסעדות וקפה</t>
+        </is>
+      </c>
+      <c r="B13" s="70" t="n">
+        <v>811</v>
+      </c>
+      <c r="C13" s="69" t="n">
+        <v>200</v>
+      </c>
+      <c r="D13" s="109" t="n">
+        <v>-611</v>
+      </c>
+      <c r="E13" s="111" t="inlineStr">
+        <is>
+          <t>⚠️ הוצאת 811₪! הגבל ל-200₪ — בשל, תכין אוכל</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="n"/>
+      <c r="G13" s="2" t="n"/>
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="n"/>
+      <c r="J13" s="2" t="n"/>
+      <c r="K13" s="2" t="n"/>
+      <c r="L13" s="2" t="n"/>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="63" t="inlineStr">
+        <is>
+          <t>🚗 תחבורה</t>
+        </is>
+      </c>
+      <c r="B14" s="112" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="64" t="n">
+        <v>150</v>
+      </c>
+      <c r="D14" s="113" t="n">
+        <v>150</v>
+      </c>
+      <c r="E14" s="110" t="inlineStr">
+        <is>
+          <t>לא הוצאת — האם יש לך נסיעות?</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="n"/>
+      <c r="G14" s="2" t="n"/>
+      <c r="H14" s="2" t="n"/>
+      <c r="I14" s="2" t="n"/>
+      <c r="J14" s="2" t="n"/>
+      <c r="K14" s="2" t="n"/>
+      <c r="L14" s="2" t="n"/>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="68" t="inlineStr">
+        <is>
+          <t>🎮 בילויים</t>
+        </is>
+      </c>
+      <c r="B15" s="114" t="n">
+        <v>66</v>
+      </c>
+      <c r="C15" s="69" t="n">
+        <v>150</v>
+      </c>
+      <c r="D15" s="113" t="n">
+        <v>84</v>
+      </c>
+      <c r="E15" s="111" t="inlineStr">
+        <is>
+          <t>✅ 66₪ — סביר</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="n"/>
+      <c r="G15" s="2" t="n"/>
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="2" t="n"/>
+      <c r="J15" s="2" t="n"/>
+      <c r="K15" s="2" t="n"/>
+      <c r="L15" s="2" t="n"/>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="63" t="inlineStr">
+        <is>
+          <t>🏥 בריאות ורפואה</t>
+        </is>
+      </c>
+      <c r="B16" s="65" t="n">
+        <v>120</v>
+      </c>
+      <c r="C16" s="64" t="n">
+        <v>80</v>
+      </c>
+      <c r="D16" s="109" t="n">
+        <v>-40</v>
+      </c>
+      <c r="E16" s="110" t="inlineStr">
+        <is>
+          <t>✅ 120₪ — סביר</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="n"/>
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="n"/>
+      <c r="J16" s="2" t="n"/>
+      <c r="K16" s="2" t="n"/>
+      <c r="L16" s="2" t="n"/>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="68" t="inlineStr">
+        <is>
+          <t>👕 ביגוד והנעלה</t>
+        </is>
+      </c>
+      <c r="B17" s="114" t="n">
+        <v>31</v>
+      </c>
+      <c r="C17" s="69" t="n">
+        <v>100</v>
+      </c>
+      <c r="D17" s="113" t="n">
+        <v>69</v>
+      </c>
+      <c r="E17" s="111" t="inlineStr">
+        <is>
+          <t>✅ 31₪ — מצוין</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="n"/>
+      <c r="G17" s="2" t="n"/>
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="2" t="n"/>
+      <c r="J17" s="2" t="n"/>
+      <c r="K17" s="2" t="n"/>
+      <c r="L17" s="2" t="n"/>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="63" t="inlineStr">
+        <is>
+          <t>📋 חשבונות קבועים</t>
+        </is>
+      </c>
+      <c r="B18" s="65" t="n">
+        <v>203</v>
+      </c>
+      <c r="C18" s="64" t="n">
+        <v>200</v>
+      </c>
+      <c r="D18" s="109" t="n">
+        <v>-3</v>
+      </c>
+      <c r="E18" s="110" t="inlineStr">
+        <is>
+          <t>שקול לבטל ChatGPT (71₪) — חסוך 71₪/חודש</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="n"/>
+      <c r="G18" s="2" t="n"/>
+      <c r="H18" s="2" t="n"/>
+      <c r="I18" s="2" t="n"/>
+      <c r="J18" s="2" t="n"/>
+      <c r="K18" s="2" t="n"/>
+      <c r="L18" s="2" t="n"/>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="68" t="inlineStr">
+        <is>
+          <t>💪 ספורט</t>
+        </is>
+      </c>
+      <c r="B19" s="114" t="n">
+        <v>600</v>
+      </c>
+      <c r="C19" s="69" t="n">
+        <v>600</v>
+      </c>
+      <c r="D19" s="113" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="111" t="inlineStr">
+        <is>
+          <t>מאמן אישי — 600₪ קבוע</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="n"/>
+      <c r="G19" s="2" t="n"/>
+      <c r="H19" s="2" t="n"/>
+      <c r="I19" s="2" t="n"/>
+      <c r="J19" s="2" t="n"/>
+      <c r="K19" s="2" t="n"/>
+      <c r="L19" s="2" t="n"/>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="63" t="inlineStr">
+        <is>
+          <t>💰 חיסכון</t>
+        </is>
+      </c>
+      <c r="B20" s="112" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="64" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D20" s="113" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E20" s="110" t="inlineStr">
+        <is>
+          <t>💰 הפרש 1,000₪ אוטומטית ב-1 לחודש!</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="n"/>
+      <c r="G20" s="2" t="n"/>
+      <c r="H20" s="2" t="n"/>
+      <c r="I20" s="2" t="n"/>
+      <c r="J20" s="2" t="n"/>
+      <c r="K20" s="2" t="n"/>
+      <c r="L20" s="2" t="n"/>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="68" t="inlineStr">
+        <is>
+          <t>🎁 מתנות</t>
+        </is>
+      </c>
+      <c r="B21" s="70" t="n">
+        <v>860</v>
+      </c>
+      <c r="C21" s="69" t="n">
+        <v>200</v>
+      </c>
+      <c r="D21" s="109" t="n">
+        <v>-660</v>
+      </c>
+      <c r="E21" s="111" t="inlineStr">
+        <is>
+          <t>⚠️ 860₪ החודש! הגדר 200₪ תקרה לחודש הבא</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="n"/>
+      <c r="G21" s="2" t="n"/>
+      <c r="H21" s="2" t="n"/>
+      <c r="I21" s="2" t="n"/>
+      <c r="J21" s="2" t="n"/>
+      <c r="K21" s="2" t="n"/>
+      <c r="L21" s="2" t="n"/>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="63" t="inlineStr">
+        <is>
+          <t>📚 חינוך</t>
+        </is>
+      </c>
+      <c r="B22" s="65" t="n">
+        <v>1100</v>
+      </c>
+      <c r="C22" s="64" t="n">
+        <v>300</v>
+      </c>
+      <c r="D22" s="109" t="n">
+        <v>-800</v>
+      </c>
+      <c r="E22" s="110" t="inlineStr">
+        <is>
+          <t>שיעורי נהיגה — כמה עוד נשארו לך לבחינה?</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="n"/>
+      <c r="G22" s="2" t="n"/>
+      <c r="H22" s="2" t="n"/>
+      <c r="I22" s="2" t="n"/>
+      <c r="J22" s="2" t="n"/>
+      <c r="K22" s="2" t="n"/>
+      <c r="L22" s="2" t="n"/>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="68" t="inlineStr">
+        <is>
+          <t>💳 אחר</t>
+        </is>
+      </c>
+      <c r="B23" s="70" t="n">
+        <v>923</v>
+      </c>
+      <c r="C23" s="69" t="n">
+        <v>150</v>
+      </c>
+      <c r="D23" s="109" t="n">
+        <v>-773</v>
+      </c>
+      <c r="E23" s="111" t="inlineStr">
+        <is>
+          <t>⚠️ 923₪! בדוק מה היה שם ותכנן מראש</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="n"/>
+      <c r="G23" s="2" t="n"/>
+      <c r="H23" s="2" t="n"/>
+      <c r="I23" s="2" t="n"/>
+      <c r="J23" s="2" t="n"/>
+      <c r="K23" s="2" t="n"/>
+      <c r="L23" s="2" t="n"/>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="115" t="inlineStr">
+        <is>
+          <t>סה"כ</t>
+        </is>
+      </c>
+      <c r="B24" s="109" t="n">
+        <v>5082</v>
+      </c>
+      <c r="C24" s="116" t="n">
+        <v>3480</v>
+      </c>
+      <c r="D24" s="109" t="n">
+        <v>-1602</v>
+      </c>
+      <c r="E24" s="2" t="n"/>
+      <c r="F24" s="2" t="n"/>
+      <c r="G24" s="2" t="n"/>
+      <c r="H24" s="2" t="n"/>
+      <c r="I24" s="2" t="n"/>
+      <c r="J24" s="2" t="n"/>
+      <c r="K24" s="2" t="n"/>
+      <c r="L24" s="2" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n"/>
+      <c r="B25" s="2" t="n"/>
+      <c r="C25" s="2" t="n"/>
+      <c r="D25" s="2" t="n"/>
+      <c r="E25" s="2" t="n"/>
+      <c r="F25" s="2" t="n"/>
+      <c r="G25" s="2" t="n"/>
+      <c r="H25" s="2" t="n"/>
+      <c r="I25" s="2" t="n"/>
+      <c r="J25" s="2" t="n"/>
+      <c r="K25" s="2" t="n"/>
+      <c r="L25" s="2" t="n"/>
+    </row>
+    <row r="26" ht="35" customHeight="1">
+      <c r="A26" s="117" t="inlineStr">
+        <is>
+          <t>🎯  יעד חיסכון חודשי: 1,000₪  |  הוראת קבע אוטומטית ב-1 לחודש!</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n"/>
+      <c r="B27" s="2" t="n"/>
+      <c r="C27" s="2" t="n"/>
+      <c r="D27" s="2" t="n"/>
+      <c r="E27" s="2" t="n"/>
+      <c r="F27" s="2" t="n"/>
+      <c r="G27" s="2" t="n"/>
+      <c r="H27" s="2" t="n"/>
+      <c r="I27" s="2" t="n"/>
+      <c r="J27" s="2" t="n"/>
+      <c r="K27" s="2" t="n"/>
+      <c r="L27" s="2" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n"/>
+      <c r="B28" s="2" t="n"/>
+      <c r="C28" s="2" t="n"/>
+      <c r="D28" s="2" t="n"/>
+      <c r="E28" s="2" t="n"/>
+      <c r="F28" s="2" t="n"/>
+      <c r="G28" s="2" t="n"/>
+      <c r="H28" s="2" t="n"/>
+      <c r="I28" s="2" t="n"/>
+      <c r="J28" s="2" t="n"/>
+      <c r="K28" s="2" t="n"/>
+      <c r="L28" s="2" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n"/>
+      <c r="B29" s="2" t="n"/>
+      <c r="C29" s="2" t="n"/>
+      <c r="D29" s="2" t="n"/>
+      <c r="E29" s="2" t="n"/>
+      <c r="F29" s="2" t="n"/>
+      <c r="G29" s="2" t="n"/>
+      <c r="H29" s="2" t="n"/>
+      <c r="I29" s="2" t="n"/>
+      <c r="J29" s="2" t="n"/>
+      <c r="K29" s="2" t="n"/>
+      <c r="L29" s="2" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n"/>
+      <c r="B30" s="2" t="n"/>
+      <c r="C30" s="2" t="n"/>
+      <c r="D30" s="2" t="n"/>
+      <c r="E30" s="2" t="n"/>
+      <c r="F30" s="2" t="n"/>
+      <c r="G30" s="2" t="n"/>
+      <c r="H30" s="2" t="n"/>
+      <c r="I30" s="2" t="n"/>
+      <c r="J30" s="2" t="n"/>
+      <c r="K30" s="2" t="n"/>
+      <c r="L30" s="2" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n"/>
+      <c r="B31" s="2" t="n"/>
+      <c r="C31" s="2" t="n"/>
+      <c r="D31" s="2" t="n"/>
+      <c r="E31" s="2" t="n"/>
+      <c r="F31" s="2" t="n"/>
+      <c r="G31" s="2" t="n"/>
+      <c r="H31" s="2" t="n"/>
+      <c r="I31" s="2" t="n"/>
+      <c r="J31" s="2" t="n"/>
+      <c r="K31" s="2" t="n"/>
+      <c r="L31" s="2" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n"/>
+      <c r="B32" s="2" t="n"/>
+      <c r="C32" s="2" t="n"/>
+      <c r="D32" s="2" t="n"/>
+      <c r="E32" s="2" t="n"/>
+      <c r="F32" s="2" t="n"/>
+      <c r="G32" s="2" t="n"/>
+      <c r="H32" s="2" t="n"/>
+      <c r="I32" s="2" t="n"/>
+      <c r="J32" s="2" t="n"/>
+      <c r="K32" s="2" t="n"/>
+      <c r="L32" s="2" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n"/>
+      <c r="B33" s="2" t="n"/>
+      <c r="C33" s="2" t="n"/>
+      <c r="D33" s="2" t="n"/>
+      <c r="E33" s="2" t="n"/>
+      <c r="F33" s="2" t="n"/>
+      <c r="G33" s="2" t="n"/>
+      <c r="H33" s="2" t="n"/>
+      <c r="I33" s="2" t="n"/>
+      <c r="J33" s="2" t="n"/>
+      <c r="K33" s="2" t="n"/>
+      <c r="L33" s="2" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n"/>
+      <c r="B34" s="2" t="n"/>
+      <c r="C34" s="2" t="n"/>
+      <c r="D34" s="2" t="n"/>
+      <c r="E34" s="2" t="n"/>
+      <c r="F34" s="2" t="n"/>
+      <c r="G34" s="2" t="n"/>
+      <c r="H34" s="2" t="n"/>
+      <c r="I34" s="2" t="n"/>
+      <c r="J34" s="2" t="n"/>
+      <c r="K34" s="2" t="n"/>
+      <c r="L34" s="2" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n"/>
+      <c r="B35" s="2" t="n"/>
+      <c r="C35" s="2" t="n"/>
+      <c r="D35" s="2" t="n"/>
+      <c r="E35" s="2" t="n"/>
+      <c r="F35" s="2" t="n"/>
+      <c r="G35" s="2" t="n"/>
+      <c r="H35" s="2" t="n"/>
+      <c r="I35" s="2" t="n"/>
+      <c r="J35" s="2" t="n"/>
+      <c r="K35" s="2" t="n"/>
+      <c r="L35" s="2" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n"/>
+      <c r="B36" s="2" t="n"/>
+      <c r="C36" s="2" t="n"/>
+      <c r="D36" s="2" t="n"/>
+      <c r="E36" s="2" t="n"/>
+      <c r="F36" s="2" t="n"/>
+      <c r="G36" s="2" t="n"/>
+      <c r="H36" s="2" t="n"/>
+      <c r="I36" s="2" t="n"/>
+      <c r="J36" s="2" t="n"/>
+      <c r="K36" s="2" t="n"/>
+      <c r="L36" s="2" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n"/>
+      <c r="B37" s="2" t="n"/>
+      <c r="C37" s="2" t="n"/>
+      <c r="D37" s="2" t="n"/>
+      <c r="E37" s="2" t="n"/>
+      <c r="F37" s="2" t="n"/>
+      <c r="G37" s="2" t="n"/>
+      <c r="H37" s="2" t="n"/>
+      <c r="I37" s="2" t="n"/>
+      <c r="J37" s="2" t="n"/>
+      <c r="K37" s="2" t="n"/>
+      <c r="L37" s="2" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n"/>
+      <c r="B38" s="2" t="n"/>
+      <c r="C38" s="2" t="n"/>
+      <c r="D38" s="2" t="n"/>
+      <c r="E38" s="2" t="n"/>
+      <c r="F38" s="2" t="n"/>
+      <c r="G38" s="2" t="n"/>
+      <c r="H38" s="2" t="n"/>
+      <c r="I38" s="2" t="n"/>
+      <c r="J38" s="2" t="n"/>
+      <c r="K38" s="2" t="n"/>
+      <c r="L38" s="2" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n"/>
+      <c r="B39" s="2" t="n"/>
+      <c r="C39" s="2" t="n"/>
+      <c r="D39" s="2" t="n"/>
+      <c r="E39" s="2" t="n"/>
+      <c r="F39" s="2" t="n"/>
+      <c r="G39" s="2" t="n"/>
+      <c r="H39" s="2" t="n"/>
+      <c r="I39" s="2" t="n"/>
+      <c r="J39" s="2" t="n"/>
+      <c r="K39" s="2" t="n"/>
+      <c r="L39" s="2" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n"/>
+      <c r="B40" s="2" t="n"/>
+      <c r="C40" s="2" t="n"/>
+      <c r="D40" s="2" t="n"/>
+      <c r="E40" s="2" t="n"/>
+      <c r="F40" s="2" t="n"/>
+      <c r="G40" s="2" t="n"/>
+      <c r="H40" s="2" t="n"/>
+      <c r="I40" s="2" t="n"/>
+      <c r="J40" s="2" t="n"/>
+      <c r="K40" s="2" t="n"/>
+      <c r="L40" s="2" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n"/>
+      <c r="B41" s="2" t="n"/>
+      <c r="C41" s="2" t="n"/>
+      <c r="D41" s="2" t="n"/>
+      <c r="E41" s="2" t="n"/>
+      <c r="F41" s="2" t="n"/>
+      <c r="G41" s="2" t="n"/>
+      <c r="H41" s="2" t="n"/>
+      <c r="I41" s="2" t="n"/>
+      <c r="J41" s="2" t="n"/>
+      <c r="K41" s="2" t="n"/>
+      <c r="L41" s="2" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n"/>
+      <c r="B42" s="2" t="n"/>
+      <c r="C42" s="2" t="n"/>
+      <c r="D42" s="2" t="n"/>
+      <c r="E42" s="2" t="n"/>
+      <c r="F42" s="2" t="n"/>
+      <c r="G42" s="2" t="n"/>
+      <c r="H42" s="2" t="n"/>
+      <c r="I42" s="2" t="n"/>
+      <c r="J42" s="2" t="n"/>
+      <c r="K42" s="2" t="n"/>
+      <c r="L42" s="2" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n"/>
+      <c r="B43" s="2" t="n"/>
+      <c r="C43" s="2" t="n"/>
+      <c r="D43" s="2" t="n"/>
+      <c r="E43" s="2" t="n"/>
+      <c r="F43" s="2" t="n"/>
+      <c r="G43" s="2" t="n"/>
+      <c r="H43" s="2" t="n"/>
+      <c r="I43" s="2" t="n"/>
+      <c r="J43" s="2" t="n"/>
+      <c r="K43" s="2" t="n"/>
+      <c r="L43" s="2" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n"/>
+      <c r="B44" s="2" t="n"/>
+      <c r="C44" s="2" t="n"/>
+      <c r="D44" s="2" t="n"/>
+      <c r="E44" s="2" t="n"/>
+      <c r="F44" s="2" t="n"/>
+      <c r="G44" s="2" t="n"/>
+      <c r="H44" s="2" t="n"/>
+      <c r="I44" s="2" t="n"/>
+      <c r="J44" s="2" t="n"/>
+      <c r="K44" s="2" t="n"/>
+      <c r="L44" s="2" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n"/>
+      <c r="B45" s="2" t="n"/>
+      <c r="C45" s="2" t="n"/>
+      <c r="D45" s="2" t="n"/>
+      <c r="E45" s="2" t="n"/>
+      <c r="F45" s="2" t="n"/>
+      <c r="G45" s="2" t="n"/>
+      <c r="H45" s="2" t="n"/>
+      <c r="I45" s="2" t="n"/>
+      <c r="J45" s="2" t="n"/>
+      <c r="K45" s="2" t="n"/>
+      <c r="L45" s="2" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n"/>
+      <c r="B46" s="2" t="n"/>
+      <c r="C46" s="2" t="n"/>
+      <c r="D46" s="2" t="n"/>
+      <c r="E46" s="2" t="n"/>
+      <c r="F46" s="2" t="n"/>
+      <c r="G46" s="2" t="n"/>
+      <c r="H46" s="2" t="n"/>
+      <c r="I46" s="2" t="n"/>
+      <c r="J46" s="2" t="n"/>
+      <c r="K46" s="2" t="n"/>
+      <c r="L46" s="2" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n"/>
+      <c r="B47" s="2" t="n"/>
+      <c r="C47" s="2" t="n"/>
+      <c r="D47" s="2" t="n"/>
+      <c r="E47" s="2" t="n"/>
+      <c r="F47" s="2" t="n"/>
+      <c r="G47" s="2" t="n"/>
+      <c r="H47" s="2" t="n"/>
+      <c r="I47" s="2" t="n"/>
+      <c r="J47" s="2" t="n"/>
+      <c r="K47" s="2" t="n"/>
+      <c r="L47" s="2" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n"/>
+      <c r="B48" s="2" t="n"/>
+      <c r="C48" s="2" t="n"/>
+      <c r="D48" s="2" t="n"/>
+      <c r="E48" s="2" t="n"/>
+      <c r="F48" s="2" t="n"/>
+      <c r="G48" s="2" t="n"/>
+      <c r="H48" s="2" t="n"/>
+      <c r="I48" s="2" t="n"/>
+      <c r="J48" s="2" t="n"/>
+      <c r="K48" s="2" t="n"/>
+      <c r="L48" s="2" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n"/>
+      <c r="B49" s="2" t="n"/>
+      <c r="C49" s="2" t="n"/>
+      <c r="D49" s="2" t="n"/>
+      <c r="E49" s="2" t="n"/>
+      <c r="F49" s="2" t="n"/>
+      <c r="G49" s="2" t="n"/>
+      <c r="H49" s="2" t="n"/>
+      <c r="I49" s="2" t="n"/>
+      <c r="J49" s="2" t="n"/>
+      <c r="K49" s="2" t="n"/>
+      <c r="L49" s="2" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n"/>
+      <c r="B50" s="2" t="n"/>
+      <c r="C50" s="2" t="n"/>
+      <c r="D50" s="2" t="n"/>
+      <c r="E50" s="2" t="n"/>
+      <c r="F50" s="2" t="n"/>
+      <c r="G50" s="2" t="n"/>
+      <c r="H50" s="2" t="n"/>
+      <c r="I50" s="2" t="n"/>
+      <c r="J50" s="2" t="n"/>
+      <c r="K50" s="2" t="n"/>
+      <c r="L50" s="2" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n"/>
+      <c r="B51" s="2" t="n"/>
+      <c r="C51" s="2" t="n"/>
+      <c r="D51" s="2" t="n"/>
+      <c r="E51" s="2" t="n"/>
+      <c r="F51" s="2" t="n"/>
+      <c r="G51" s="2" t="n"/>
+      <c r="H51" s="2" t="n"/>
+      <c r="I51" s="2" t="n"/>
+      <c r="J51" s="2" t="n"/>
+      <c r="K51" s="2" t="n"/>
+      <c r="L51" s="2" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n"/>
+      <c r="B52" s="2" t="n"/>
+      <c r="C52" s="2" t="n"/>
+      <c r="D52" s="2" t="n"/>
+      <c r="E52" s="2" t="n"/>
+      <c r="F52" s="2" t="n"/>
+      <c r="G52" s="2" t="n"/>
+      <c r="H52" s="2" t="n"/>
+      <c r="I52" s="2" t="n"/>
+      <c r="J52" s="2" t="n"/>
+      <c r="K52" s="2" t="n"/>
+      <c r="L52" s="2" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n"/>
+      <c r="B53" s="2" t="n"/>
+      <c r="C53" s="2" t="n"/>
+      <c r="D53" s="2" t="n"/>
+      <c r="E53" s="2" t="n"/>
+      <c r="F53" s="2" t="n"/>
+      <c r="G53" s="2" t="n"/>
+      <c r="H53" s="2" t="n"/>
+      <c r="I53" s="2" t="n"/>
+      <c r="J53" s="2" t="n"/>
+      <c r="K53" s="2" t="n"/>
+      <c r="L53" s="2" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n"/>
+      <c r="B54" s="2" t="n"/>
+      <c r="C54" s="2" t="n"/>
+      <c r="D54" s="2" t="n"/>
+      <c r="E54" s="2" t="n"/>
+      <c r="F54" s="2" t="n"/>
+      <c r="G54" s="2" t="n"/>
+      <c r="H54" s="2" t="n"/>
+      <c r="I54" s="2" t="n"/>
+      <c r="J54" s="2" t="n"/>
+      <c r="K54" s="2" t="n"/>
+      <c r="L54" s="2" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n"/>
+      <c r="B55" s="2" t="n"/>
+      <c r="C55" s="2" t="n"/>
+      <c r="D55" s="2" t="n"/>
+      <c r="E55" s="2" t="n"/>
+      <c r="F55" s="2" t="n"/>
+      <c r="G55" s="2" t="n"/>
+      <c r="H55" s="2" t="n"/>
+      <c r="I55" s="2" t="n"/>
+      <c r="J55" s="2" t="n"/>
+      <c r="K55" s="2" t="n"/>
+      <c r="L55" s="2" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n"/>
+      <c r="B56" s="2" t="n"/>
+      <c r="C56" s="2" t="n"/>
+      <c r="D56" s="2" t="n"/>
+      <c r="E56" s="2" t="n"/>
+      <c r="F56" s="2" t="n"/>
+      <c r="G56" s="2" t="n"/>
+      <c r="H56" s="2" t="n"/>
+      <c r="I56" s="2" t="n"/>
+      <c r="J56" s="2" t="n"/>
+      <c r="K56" s="2" t="n"/>
+      <c r="L56" s="2" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n"/>
+      <c r="B57" s="2" t="n"/>
+      <c r="C57" s="2" t="n"/>
+      <c r="D57" s="2" t="n"/>
+      <c r="E57" s="2" t="n"/>
+      <c r="F57" s="2" t="n"/>
+      <c r="G57" s="2" t="n"/>
+      <c r="H57" s="2" t="n"/>
+      <c r="I57" s="2" t="n"/>
+      <c r="J57" s="2" t="n"/>
+      <c r="K57" s="2" t="n"/>
+      <c r="L57" s="2" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n"/>
+      <c r="B58" s="2" t="n"/>
+      <c r="C58" s="2" t="n"/>
+      <c r="D58" s="2" t="n"/>
+      <c r="E58" s="2" t="n"/>
+      <c r="F58" s="2" t="n"/>
+      <c r="G58" s="2" t="n"/>
+      <c r="H58" s="2" t="n"/>
+      <c r="I58" s="2" t="n"/>
+      <c r="J58" s="2" t="n"/>
+      <c r="K58" s="2" t="n"/>
+      <c r="L58" s="2" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n"/>
+      <c r="B59" s="2" t="n"/>
+      <c r="C59" s="2" t="n"/>
+      <c r="D59" s="2" t="n"/>
+      <c r="E59" s="2" t="n"/>
+      <c r="F59" s="2" t="n"/>
+      <c r="G59" s="2" t="n"/>
+      <c r="H59" s="2" t="n"/>
+      <c r="I59" s="2" t="n"/>
+      <c r="J59" s="2" t="n"/>
+      <c r="K59" s="2" t="n"/>
+      <c r="L59" s="2" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n"/>
+      <c r="B60" s="2" t="n"/>
+      <c r="C60" s="2" t="n"/>
+      <c r="D60" s="2" t="n"/>
+      <c r="E60" s="2" t="n"/>
+      <c r="F60" s="2" t="n"/>
+      <c r="G60" s="2" t="n"/>
+      <c r="H60" s="2" t="n"/>
+      <c r="I60" s="2" t="n"/>
+      <c r="J60" s="2" t="n"/>
+      <c r="K60" s="2" t="n"/>
+      <c r="L60" s="2" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n"/>
+      <c r="B61" s="2" t="n"/>
+      <c r="C61" s="2" t="n"/>
+      <c r="D61" s="2" t="n"/>
+      <c r="E61" s="2" t="n"/>
+      <c r="F61" s="2" t="n"/>
+      <c r="G61" s="2" t="n"/>
+      <c r="H61" s="2" t="n"/>
+      <c r="I61" s="2" t="n"/>
+      <c r="J61" s="2" t="n"/>
+      <c r="K61" s="2" t="n"/>
+      <c r="L61" s="2" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n"/>
+      <c r="B62" s="2" t="n"/>
+      <c r="C62" s="2" t="n"/>
+      <c r="D62" s="2" t="n"/>
+      <c r="E62" s="2" t="n"/>
+      <c r="F62" s="2" t="n"/>
+      <c r="G62" s="2" t="n"/>
+      <c r="H62" s="2" t="n"/>
+      <c r="I62" s="2" t="n"/>
+      <c r="J62" s="2" t="n"/>
+      <c r="K62" s="2" t="n"/>
+      <c r="L62" s="2" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n"/>
+      <c r="B63" s="2" t="n"/>
+      <c r="C63" s="2" t="n"/>
+      <c r="D63" s="2" t="n"/>
+      <c r="E63" s="2" t="n"/>
+      <c r="F63" s="2" t="n"/>
+      <c r="G63" s="2" t="n"/>
+      <c r="H63" s="2" t="n"/>
+      <c r="I63" s="2" t="n"/>
+      <c r="J63" s="2" t="n"/>
+      <c r="K63" s="2" t="n"/>
+      <c r="L63" s="2" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n"/>
+      <c r="B64" s="2" t="n"/>
+      <c r="C64" s="2" t="n"/>
+      <c r="D64" s="2" t="n"/>
+      <c r="E64" s="2" t="n"/>
+      <c r="F64" s="2" t="n"/>
+      <c r="G64" s="2" t="n"/>
+      <c r="H64" s="2" t="n"/>
+      <c r="I64" s="2" t="n"/>
+      <c r="J64" s="2" t="n"/>
+      <c r="K64" s="2" t="n"/>
+      <c r="L64" s="2" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n"/>
+      <c r="B65" s="2" t="n"/>
+      <c r="C65" s="2" t="n"/>
+      <c r="D65" s="2" t="n"/>
+      <c r="E65" s="2" t="n"/>
+      <c r="F65" s="2" t="n"/>
+      <c r="G65" s="2" t="n"/>
+      <c r="H65" s="2" t="n"/>
+      <c r="I65" s="2" t="n"/>
+      <c r="J65" s="2" t="n"/>
+      <c r="K65" s="2" t="n"/>
+      <c r="L65" s="2" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n"/>
+      <c r="B66" s="2" t="n"/>
+      <c r="C66" s="2" t="n"/>
+      <c r="D66" s="2" t="n"/>
+      <c r="E66" s="2" t="n"/>
+      <c r="F66" s="2" t="n"/>
+      <c r="G66" s="2" t="n"/>
+      <c r="H66" s="2" t="n"/>
+      <c r="I66" s="2" t="n"/>
+      <c r="J66" s="2" t="n"/>
+      <c r="K66" s="2" t="n"/>
+      <c r="L66" s="2" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n"/>
+      <c r="B67" s="2" t="n"/>
+      <c r="C67" s="2" t="n"/>
+      <c r="D67" s="2" t="n"/>
+      <c r="E67" s="2" t="n"/>
+      <c r="F67" s="2" t="n"/>
+      <c r="G67" s="2" t="n"/>
+      <c r="H67" s="2" t="n"/>
+      <c r="I67" s="2" t="n"/>
+      <c r="J67" s="2" t="n"/>
+      <c r="K67" s="2" t="n"/>
+      <c r="L67" s="2" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n"/>
+      <c r="B68" s="2" t="n"/>
+      <c r="C68" s="2" t="n"/>
+      <c r="D68" s="2" t="n"/>
+      <c r="E68" s="2" t="n"/>
+      <c r="F68" s="2" t="n"/>
+      <c r="G68" s="2" t="n"/>
+      <c r="H68" s="2" t="n"/>
+      <c r="I68" s="2" t="n"/>
+      <c r="J68" s="2" t="n"/>
+      <c r="K68" s="2" t="n"/>
+      <c r="L68" s="2" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n"/>
+      <c r="B69" s="2" t="n"/>
+      <c r="C69" s="2" t="n"/>
+      <c r="D69" s="2" t="n"/>
+      <c r="E69" s="2" t="n"/>
+      <c r="F69" s="2" t="n"/>
+      <c r="G69" s="2" t="n"/>
+      <c r="H69" s="2" t="n"/>
+      <c r="I69" s="2" t="n"/>
+      <c r="J69" s="2" t="n"/>
+      <c r="K69" s="2" t="n"/>
+      <c r="L69" s="2" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n"/>
+      <c r="B70" s="2" t="n"/>
+      <c r="C70" s="2" t="n"/>
+      <c r="D70" s="2" t="n"/>
+      <c r="E70" s="2" t="n"/>
+      <c r="F70" s="2" t="n"/>
+      <c r="G70" s="2" t="n"/>
+      <c r="H70" s="2" t="n"/>
+      <c r="I70" s="2" t="n"/>
+      <c r="J70" s="2" t="n"/>
+      <c r="K70" s="2" t="n"/>
+      <c r="L70" s="2" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n"/>
+      <c r="B71" s="2" t="n"/>
+      <c r="C71" s="2" t="n"/>
+      <c r="D71" s="2" t="n"/>
+      <c r="E71" s="2" t="n"/>
+      <c r="F71" s="2" t="n"/>
+      <c r="G71" s="2" t="n"/>
+      <c r="H71" s="2" t="n"/>
+      <c r="I71" s="2" t="n"/>
+      <c r="J71" s="2" t="n"/>
+      <c r="K71" s="2" t="n"/>
+      <c r="L71" s="2" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n"/>
+      <c r="B72" s="2" t="n"/>
+      <c r="C72" s="2" t="n"/>
+      <c r="D72" s="2" t="n"/>
+      <c r="E72" s="2" t="n"/>
+      <c r="F72" s="2" t="n"/>
+      <c r="G72" s="2" t="n"/>
+      <c r="H72" s="2" t="n"/>
+      <c r="I72" s="2" t="n"/>
+      <c r="J72" s="2" t="n"/>
+      <c r="K72" s="2" t="n"/>
+      <c r="L72" s="2" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n"/>
+      <c r="B73" s="2" t="n"/>
+      <c r="C73" s="2" t="n"/>
+      <c r="D73" s="2" t="n"/>
+      <c r="E73" s="2" t="n"/>
+      <c r="F73" s="2" t="n"/>
+      <c r="G73" s="2" t="n"/>
+      <c r="H73" s="2" t="n"/>
+      <c r="I73" s="2" t="n"/>
+      <c r="J73" s="2" t="n"/>
+      <c r="K73" s="2" t="n"/>
+      <c r="L73" s="2" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n"/>
+      <c r="B74" s="2" t="n"/>
+      <c r="C74" s="2" t="n"/>
+      <c r="D74" s="2" t="n"/>
+      <c r="E74" s="2" t="n"/>
+      <c r="F74" s="2" t="n"/>
+      <c r="G74" s="2" t="n"/>
+      <c r="H74" s="2" t="n"/>
+      <c r="I74" s="2" t="n"/>
+      <c r="J74" s="2" t="n"/>
+      <c r="K74" s="2" t="n"/>
+      <c r="L74" s="2" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n"/>
+      <c r="B75" s="2" t="n"/>
+      <c r="C75" s="2" t="n"/>
+      <c r="D75" s="2" t="n"/>
+      <c r="E75" s="2" t="n"/>
+      <c r="F75" s="2" t="n"/>
+      <c r="G75" s="2" t="n"/>
+      <c r="H75" s="2" t="n"/>
+      <c r="I75" s="2" t="n"/>
+      <c r="J75" s="2" t="n"/>
+      <c r="K75" s="2" t="n"/>
+      <c r="L75" s="2" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n"/>
+      <c r="B76" s="2" t="n"/>
+      <c r="C76" s="2" t="n"/>
+      <c r="D76" s="2" t="n"/>
+      <c r="E76" s="2" t="n"/>
+      <c r="F76" s="2" t="n"/>
+      <c r="G76" s="2" t="n"/>
+      <c r="H76" s="2" t="n"/>
+      <c r="I76" s="2" t="n"/>
+      <c r="J76" s="2" t="n"/>
+      <c r="K76" s="2" t="n"/>
+      <c r="L76" s="2" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n"/>
+      <c r="B77" s="2" t="n"/>
+      <c r="C77" s="2" t="n"/>
+      <c r="D77" s="2" t="n"/>
+      <c r="E77" s="2" t="n"/>
+      <c r="F77" s="2" t="n"/>
+      <c r="G77" s="2" t="n"/>
+      <c r="H77" s="2" t="n"/>
+      <c r="I77" s="2" t="n"/>
+      <c r="J77" s="2" t="n"/>
+      <c r="K77" s="2" t="n"/>
+      <c r="L77" s="2" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n"/>
+      <c r="B78" s="2" t="n"/>
+      <c r="C78" s="2" t="n"/>
+      <c r="D78" s="2" t="n"/>
+      <c r="E78" s="2" t="n"/>
+      <c r="F78" s="2" t="n"/>
+      <c r="G78" s="2" t="n"/>
+      <c r="H78" s="2" t="n"/>
+      <c r="I78" s="2" t="n"/>
+      <c r="J78" s="2" t="n"/>
+      <c r="K78" s="2" t="n"/>
+      <c r="L78" s="2" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n"/>
+      <c r="B79" s="2" t="n"/>
+      <c r="C79" s="2" t="n"/>
+      <c r="D79" s="2" t="n"/>
+      <c r="E79" s="2" t="n"/>
+      <c r="F79" s="2" t="n"/>
+      <c r="G79" s="2" t="n"/>
+      <c r="H79" s="2" t="n"/>
+      <c r="I79" s="2" t="n"/>
+      <c r="J79" s="2" t="n"/>
+      <c r="K79" s="2" t="n"/>
+      <c r="L79" s="2" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n"/>
+      <c r="B80" s="2" t="n"/>
+      <c r="C80" s="2" t="n"/>
+      <c r="D80" s="2" t="n"/>
+      <c r="E80" s="2" t="n"/>
+      <c r="F80" s="2" t="n"/>
+      <c r="G80" s="2" t="n"/>
+      <c r="H80" s="2" t="n"/>
+      <c r="I80" s="2" t="n"/>
+      <c r="J80" s="2" t="n"/>
+      <c r="K80" s="2" t="n"/>
+      <c r="L80" s="2" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n"/>
+      <c r="B81" s="2" t="n"/>
+      <c r="C81" s="2" t="n"/>
+      <c r="D81" s="2" t="n"/>
+      <c r="E81" s="2" t="n"/>
+      <c r="F81" s="2" t="n"/>
+      <c r="G81" s="2" t="n"/>
+      <c r="H81" s="2" t="n"/>
+      <c r="I81" s="2" t="n"/>
+      <c r="J81" s="2" t="n"/>
+      <c r="K81" s="2" t="n"/>
+      <c r="L81" s="2" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n"/>
+      <c r="B82" s="2" t="n"/>
+      <c r="C82" s="2" t="n"/>
+      <c r="D82" s="2" t="n"/>
+      <c r="E82" s="2" t="n"/>
+      <c r="F82" s="2" t="n"/>
+      <c r="G82" s="2" t="n"/>
+      <c r="H82" s="2" t="n"/>
+      <c r="I82" s="2" t="n"/>
+      <c r="J82" s="2" t="n"/>
+      <c r="K82" s="2" t="n"/>
+      <c r="L82" s="2" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n"/>
+      <c r="B83" s="2" t="n"/>
+      <c r="C83" s="2" t="n"/>
+      <c r="D83" s="2" t="n"/>
+      <c r="E83" s="2" t="n"/>
+      <c r="F83" s="2" t="n"/>
+      <c r="G83" s="2" t="n"/>
+      <c r="H83" s="2" t="n"/>
+      <c r="I83" s="2" t="n"/>
+      <c r="J83" s="2" t="n"/>
+      <c r="K83" s="2" t="n"/>
+      <c r="L83" s="2" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n"/>
+      <c r="B84" s="2" t="n"/>
+      <c r="C84" s="2" t="n"/>
+      <c r="D84" s="2" t="n"/>
+      <c r="E84" s="2" t="n"/>
+      <c r="F84" s="2" t="n"/>
+      <c r="G84" s="2" t="n"/>
+      <c r="H84" s="2" t="n"/>
+      <c r="I84" s="2" t="n"/>
+      <c r="J84" s="2" t="n"/>
+      <c r="K84" s="2" t="n"/>
+      <c r="L84" s="2" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n"/>
+      <c r="B85" s="2" t="n"/>
+      <c r="C85" s="2" t="n"/>
+      <c r="D85" s="2" t="n"/>
+      <c r="E85" s="2" t="n"/>
+      <c r="F85" s="2" t="n"/>
+      <c r="G85" s="2" t="n"/>
+      <c r="H85" s="2" t="n"/>
+      <c r="I85" s="2" t="n"/>
+      <c r="J85" s="2" t="n"/>
+      <c r="K85" s="2" t="n"/>
+      <c r="L85" s="2" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n"/>
+      <c r="B86" s="2" t="n"/>
+      <c r="C86" s="2" t="n"/>
+      <c r="D86" s="2" t="n"/>
+      <c r="E86" s="2" t="n"/>
+      <c r="F86" s="2" t="n"/>
+      <c r="G86" s="2" t="n"/>
+      <c r="H86" s="2" t="n"/>
+      <c r="I86" s="2" t="n"/>
+      <c r="J86" s="2" t="n"/>
+      <c r="K86" s="2" t="n"/>
+      <c r="L86" s="2" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n"/>
+      <c r="B87" s="2" t="n"/>
+      <c r="C87" s="2" t="n"/>
+      <c r="D87" s="2" t="n"/>
+      <c r="E87" s="2" t="n"/>
+      <c r="F87" s="2" t="n"/>
+      <c r="G87" s="2" t="n"/>
+      <c r="H87" s="2" t="n"/>
+      <c r="I87" s="2" t="n"/>
+      <c r="J87" s="2" t="n"/>
+      <c r="K87" s="2" t="n"/>
+      <c r="L87" s="2" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n"/>
+      <c r="B88" s="2" t="n"/>
+      <c r="C88" s="2" t="n"/>
+      <c r="D88" s="2" t="n"/>
+      <c r="E88" s="2" t="n"/>
+      <c r="F88" s="2" t="n"/>
+      <c r="G88" s="2" t="n"/>
+      <c r="H88" s="2" t="n"/>
+      <c r="I88" s="2" t="n"/>
+      <c r="J88" s="2" t="n"/>
+      <c r="K88" s="2" t="n"/>
+      <c r="L88" s="2" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n"/>
+      <c r="B89" s="2" t="n"/>
+      <c r="C89" s="2" t="n"/>
+      <c r="D89" s="2" t="n"/>
+      <c r="E89" s="2" t="n"/>
+      <c r="F89" s="2" t="n"/>
+      <c r="G89" s="2" t="n"/>
+      <c r="H89" s="2" t="n"/>
+      <c r="I89" s="2" t="n"/>
+      <c r="J89" s="2" t="n"/>
+      <c r="K89" s="2" t="n"/>
+      <c r="L89" s="2" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A26:L26"/>
+    <mergeCell ref="A10:L10"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A24"/>
+    <mergeCell ref="A3:L3"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add daily expenses 18/04: taxi 50₪ + restaurant 340₪
https://claude.ai/code/session_01Cwu7SWtx13xhFUMhTaLvjR
</commit_message>
<xml_diff>
--- a/finance/מעקב_פיננסי.xlsx
+++ b/finance/מעקב_פיננסי.xlsx
@@ -1137,7 +1137,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>עודכן לאחרונה: 18/04/2026 06:03</t>
+          <t>עודכן לאחרונה: 18/04/2026 18:44</t>
         </is>
       </c>
       <c r="Q2" s="2" t="n"/>
@@ -1203,19 +1203,19 @@
       <c r="D5" s="2" t="n"/>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>₪5,082</t>
+          <t>₪5,472</t>
         </is>
       </c>
       <c r="H5" s="2" t="n"/>
       <c r="I5" s="10" t="inlineStr">
         <is>
-          <t>₪3,996</t>
+          <t>₪3,606</t>
         </is>
       </c>
       <c r="L5" s="2" t="n"/>
       <c r="M5" s="11" t="inlineStr">
         <is>
-          <t>44.0%</t>
+          <t>39.7%</t>
         </is>
       </c>
       <c r="P5" s="2" t="n"/>
@@ -5143,27 +5143,71 @@
       <c r="J32" s="2" t="n"/>
       <c r="K32" s="2" t="n"/>
     </row>
-    <row r="33">
-      <c r="A33" s="2" t="n"/>
-      <c r="B33" s="2" t="n"/>
-      <c r="C33" s="2" t="n"/>
-      <c r="D33" s="2" t="n"/>
-      <c r="E33" s="2" t="n"/>
-      <c r="F33" s="2" t="n"/>
-      <c r="G33" s="2" t="n"/>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="39" t="inlineStr">
+        <is>
+          <t>18/04/2026</t>
+        </is>
+      </c>
+      <c r="B33" s="40" t="inlineStr">
+        <is>
+          <t>תחבורה</t>
+        </is>
+      </c>
+      <c r="C33" s="39" t="inlineStr">
+        <is>
+          <t>מונית</t>
+        </is>
+      </c>
+      <c r="D33" s="41" t="n">
+        <v>50</v>
+      </c>
+      <c r="E33" s="39" t="inlineStr">
+        <is>
+          <t>לא צוין</t>
+        </is>
+      </c>
+      <c r="F33" s="42" t="inlineStr">
+        <is>
+          <t>❌ לא</t>
+        </is>
+      </c>
+      <c r="G33" s="39" t="inlineStr"/>
       <c r="H33" s="2" t="n"/>
       <c r="I33" s="2" t="n"/>
       <c r="J33" s="2" t="n"/>
       <c r="K33" s="2" t="n"/>
     </row>
-    <row r="34">
-      <c r="A34" s="2" t="n"/>
-      <c r="B34" s="2" t="n"/>
-      <c r="C34" s="2" t="n"/>
-      <c r="D34" s="2" t="n"/>
-      <c r="E34" s="2" t="n"/>
-      <c r="F34" s="2" t="n"/>
-      <c r="G34" s="2" t="n"/>
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="43" t="inlineStr">
+        <is>
+          <t>18/04/2026</t>
+        </is>
+      </c>
+      <c r="B34" s="44" t="inlineStr">
+        <is>
+          <t>מסעדות וקפה</t>
+        </is>
+      </c>
+      <c r="C34" s="43" t="inlineStr">
+        <is>
+          <t>מסעדה</t>
+        </is>
+      </c>
+      <c r="D34" s="45" t="n">
+        <v>340</v>
+      </c>
+      <c r="E34" s="43" t="inlineStr">
+        <is>
+          <t>לא צוין</t>
+        </is>
+      </c>
+      <c r="F34" s="46" t="inlineStr">
+        <is>
+          <t>❌ לא</t>
+        </is>
+      </c>
+      <c r="G34" s="43" t="inlineStr"/>
       <c r="H34" s="2" t="n"/>
       <c r="I34" s="2" t="n"/>
       <c r="J34" s="2" t="n"/>
@@ -12532,13 +12576,13 @@
         <v>200</v>
       </c>
       <c r="C4" s="70" t="n">
-        <v>811</v>
+        <v>1151</v>
       </c>
       <c r="D4" s="71" t="n">
-        <v>-611</v>
+        <v>-951</v>
       </c>
       <c r="E4" s="72" t="n">
-        <v>4.055</v>
+        <v>5.755</v>
       </c>
       <c r="F4" s="73" t="inlineStr">
         <is>
@@ -12561,13 +12605,13 @@
         <v>150</v>
       </c>
       <c r="C5" s="74" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="D5" s="75" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="E5" s="67" t="n">
-        <v>0</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="F5" s="76" t="inlineStr">
         <is>
@@ -13801,7 +13845,7 @@
         <v>860</v>
       </c>
       <c r="C3" s="83" t="n">
-        <v>0.1692247146792601</v>
+        <v>0.1586130579122095</v>
       </c>
       <c r="D3" s="84" t="n">
         <v>47.77777777777778</v>
@@ -13828,19 +13872,19 @@
         </is>
       </c>
       <c r="B4" s="88" t="n">
-        <v>811</v>
+        <v>1151</v>
       </c>
       <c r="C4" s="89" t="n">
-        <v>0.1595828414010232</v>
+        <v>0.2122832902987827</v>
       </c>
       <c r="D4" s="90" t="n">
-        <v>45.05555555555556</v>
+        <v>63.94444444444444</v>
       </c>
       <c r="E4" s="91" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F4" s="92" t="n">
-        <v>286</v>
+        <v>340</v>
       </c>
       <c r="G4" s="2" t="n"/>
       <c r="H4" s="2" t="n"/>
@@ -13861,7 +13905,7 @@
         <v>368</v>
       </c>
       <c r="C5" s="83" t="n">
-        <v>0.07241243604879968</v>
+        <v>0.06787163408336407</v>
       </c>
       <c r="D5" s="84" t="n">
         <v>20.44444444444444</v>
@@ -13891,7 +13935,7 @@
         <v>203</v>
       </c>
       <c r="C6" s="89" t="n">
-        <v>0.03994490358126722</v>
+        <v>0.03744005901881225</v>
       </c>
       <c r="D6" s="90" t="n">
         <v>11.27777777777778</v>
@@ -13921,7 +13965,7 @@
         <v>66</v>
       </c>
       <c r="C7" s="83" t="n">
-        <v>0.01298701298701299</v>
+        <v>0.01217263002582073</v>
       </c>
       <c r="D7" s="84" t="n">
         <v>3.666666666666667</v>
@@ -13951,7 +13995,7 @@
         <v>923</v>
       </c>
       <c r="C8" s="89" t="n">
-        <v>0.1816214088941362</v>
+        <v>0.1702323865732202</v>
       </c>
       <c r="D8" s="90" t="n">
         <v>51.27777777777778</v>
@@ -13981,7 +14025,7 @@
         <v>31</v>
       </c>
       <c r="C9" s="83" t="n">
-        <v>0.006099960645415191</v>
+        <v>0.005717447436370343</v>
       </c>
       <c r="D9" s="84" t="n">
         <v>1.722222222222222</v>
@@ -14011,7 +14055,7 @@
         <v>120</v>
       </c>
       <c r="C10" s="89" t="n">
-        <v>0.02361275088547816</v>
+        <v>0.02213205459240133</v>
       </c>
       <c r="D10" s="90" t="n">
         <v>6.666666666666667</v>
@@ -14041,7 +14085,7 @@
         <v>1100</v>
       </c>
       <c r="C11" s="83" t="n">
-        <v>0.2164502164502164</v>
+        <v>0.2028771670970122</v>
       </c>
       <c r="D11" s="84" t="n">
         <v>61.11111111111111</v>
@@ -14071,7 +14115,7 @@
         <v>600</v>
       </c>
       <c r="C12" s="89" t="n">
-        <v>0.1180637544273908</v>
+        <v>0.1106602729620066</v>
       </c>
       <c r="D12" s="90" t="n">
         <v>33.33333333333334</v>
@@ -14098,7 +14142,7 @@
         </is>
       </c>
       <c r="B13" s="100" t="n">
-        <v>5082</v>
+        <v>5422</v>
       </c>
       <c r="C13" s="101" t="n">
         <v>1</v>
@@ -17191,13 +17235,13 @@
         </is>
       </c>
       <c r="B13" s="70" t="n">
-        <v>811</v>
+        <v>1151</v>
       </c>
       <c r="C13" s="69" t="n">
         <v>200</v>
       </c>
       <c r="D13" s="109" t="n">
-        <v>-611</v>
+        <v>-951</v>
       </c>
       <c r="E13" s="111" t="inlineStr">
         <is>
@@ -17219,13 +17263,13 @@
         </is>
       </c>
       <c r="B14" s="112" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="C14" s="64" t="n">
         <v>150</v>
       </c>
       <c r="D14" s="113" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="E14" s="110" t="inlineStr">
         <is>
@@ -17499,13 +17543,13 @@
         </is>
       </c>
       <c r="B24" s="109" t="n">
-        <v>5082</v>
+        <v>5472</v>
       </c>
       <c r="C24" s="116" t="n">
         <v>3480</v>
       </c>
       <c r="D24" s="109" t="n">
-        <v>-1602</v>
+        <v>-1992</v>
       </c>
       <c r="E24" s="2" t="n"/>
       <c r="F24" s="2" t="n"/>

</xml_diff>

<commit_message>
Add taxi 40₪ on 18/04, update monthly totals
https://claude.ai/code/session_01Cwu7SWtx13xhFUMhTaLvjR
</commit_message>
<xml_diff>
--- a/finance/מעקב_פיננסי.xlsx
+++ b/finance/מעקב_פיננסי.xlsx
@@ -1137,7 +1137,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>עודכן לאחרונה: 18/04/2026 18:44</t>
+          <t>עודכן לאחרונה: 18/04/2026 19:12</t>
         </is>
       </c>
       <c r="Q2" s="2" t="n"/>
@@ -1203,19 +1203,19 @@
       <c r="D5" s="2" t="n"/>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>₪5,472</t>
+          <t>₪5,512</t>
         </is>
       </c>
       <c r="H5" s="2" t="n"/>
       <c r="I5" s="10" t="inlineStr">
         <is>
-          <t>₪3,606</t>
+          <t>₪3,566</t>
         </is>
       </c>
       <c r="L5" s="2" t="n"/>
       <c r="M5" s="11" t="inlineStr">
         <is>
-          <t>39.7%</t>
+          <t>39.3%</t>
         </is>
       </c>
       <c r="P5" s="2" t="n"/>
@@ -5213,14 +5213,36 @@
       <c r="J34" s="2" t="n"/>
       <c r="K34" s="2" t="n"/>
     </row>
-    <row r="35">
-      <c r="A35" s="2" t="n"/>
-      <c r="B35" s="2" t="n"/>
-      <c r="C35" s="2" t="n"/>
-      <c r="D35" s="2" t="n"/>
-      <c r="E35" s="2" t="n"/>
-      <c r="F35" s="2" t="n"/>
-      <c r="G35" s="2" t="n"/>
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="39" t="inlineStr">
+        <is>
+          <t>18/04/2026</t>
+        </is>
+      </c>
+      <c r="B35" s="40" t="inlineStr">
+        <is>
+          <t>תחבורה</t>
+        </is>
+      </c>
+      <c r="C35" s="39" t="inlineStr">
+        <is>
+          <t>מונית</t>
+        </is>
+      </c>
+      <c r="D35" s="41" t="n">
+        <v>40</v>
+      </c>
+      <c r="E35" s="39" t="inlineStr">
+        <is>
+          <t>לא צוין</t>
+        </is>
+      </c>
+      <c r="F35" s="42" t="inlineStr">
+        <is>
+          <t>❌ לא</t>
+        </is>
+      </c>
+      <c r="G35" s="39" t="inlineStr"/>
       <c r="H35" s="2" t="n"/>
       <c r="I35" s="2" t="n"/>
       <c r="J35" s="2" t="n"/>
@@ -12605,13 +12627,13 @@
         <v>150</v>
       </c>
       <c r="C5" s="74" t="n">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="D5" s="75" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="E5" s="67" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.6</v>
       </c>
       <c r="F5" s="76" t="inlineStr">
         <is>
@@ -17263,13 +17285,13 @@
         </is>
       </c>
       <c r="B14" s="112" t="n">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="C14" s="64" t="n">
         <v>150</v>
       </c>
       <c r="D14" s="113" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="E14" s="110" t="inlineStr">
         <is>
@@ -17543,13 +17565,13 @@
         </is>
       </c>
       <c r="B24" s="109" t="n">
-        <v>5472</v>
+        <v>5512</v>
       </c>
       <c r="C24" s="116" t="n">
         <v>3480</v>
       </c>
       <c r="D24" s="109" t="n">
-        <v>-1992</v>
+        <v>-2032</v>
       </c>
       <c r="E24" s="2" t="n"/>
       <c r="F24" s="2" t="n"/>

</xml_diff>